<commit_message>
feat(admin): add account moderation and session revocation (#64)
</commit_message>
<xml_diff>
--- a/docs/requirements/UniConnect_Requirements_Baseline.xlsx
+++ b/docs/requirements/UniConnect_Requirements_Baseline.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="Rcf8013865f31425f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="R19e26ab60ec64ab8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="Rd5b7d80ce6234c46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="R5a8ebbee880d47d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="Rb897d9c835614911"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="R1031445abf4741f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="R3e3432dc7e4a4baa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Re41e933701ac4c6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="R91c5e0853a3f45fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="Rb590d7afb9534d5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="Rfaa9ca7984db4f97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="R86c04731cf3140f8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -929,7 +929,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -940,7 +940,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -951,7 +951,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -33049,7 +33049,7 @@
 - ClubStatus becomes PUBLISHING_SUSPENDED and the reason/state change is audited.
 - New Club publications are blocked.
 - The Club profile and already-published announcements remain visible.
-- If suspension resulted from an unavailable administrator, publishing cannot be restored until an eligible replacement is appointed.</x:v>
+- If suspension resulted from an unavailable administrator, restoration requires exactly one eligible current CLUB_ADMINISTRATOR. Reactivating the original administrator may satisfy eligibility, but account reactivation does not restore publishing; an authorized SYSTEM_ADMIN must explicitly restore it under FR_83.</x:v>
       </x:c>
       <x:c r="K78" s="15" t="str">
         <x:v>High</x:v>
@@ -33599,7 +33599,8 @@
         <x:v>- Only an ACTIVE SYSTEM_ADMIN may restore publishing.
 - The Club currently has status PUBLISHING_SUSPENDED.
 - A reason or resolution note is required.
-- The Club has exactly one eligible current CLUB_ADMINISTRATOR.
+- The Club has exactly one eligible current CLUB_ADMINISTRATOR; this may be the original administrator after account reactivation.
+- Account reactivation never restores Club publishing; restoration is this explicit action.
 - ClubStatus becomes ACTIVE.
 - Authorized operators may publish again.
 - The state change is recorded in immutable audit history and produces one informational notification event.</x:v>
@@ -63492,9 +63493,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f06587077094fc5"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f1b418e25df4909"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc7e3952839a4826"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb249208ad2874dda"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -65770,7 +65771,7 @@
         <x:v>Called a Club an account and treated suspension as full invisibility.</x:v>
       </x:c>
       <x:c r="H78" s="31" t="str">
-        <x:v>Used canonical ClubStatus and limited suspension to new publishing.</x:v>
+        <x:v>Used canonical ClubStatus, limited suspension to new publishing, and clarified that a reactivated original administrator may satisfy eligibility while explicit FR_83 restoration remains required.</x:v>
       </x:c>
       <x:c r="I78" s="31" t="str">
         <x:v>UniConnect_Administration_Notification_Class_Diagram_Corrected.drawio</x:v>
@@ -66031,7 +66032,7 @@
         <x:v>Restoring Club publishing existed in the administration model but had no atomic functional requirement.</x:v>
       </x:c>
       <x:c r="H87" s="30" t="str">
-        <x:v>Added an authorized, audited restoration requirement with an eligible-administrator precondition.</x:v>
+        <x:v>Added an authorized, audited explicit restoration requirement; an eligible current administrator may be the reactivated original administrator, but reactivation alone never restores publishing.</x:v>
       </x:c>
       <x:c r="I87" s="30" t="str">
         <x:v>UniConnect_Administration_Notification_Class_Diagram_Corrected.drawio</x:v>
@@ -66248,7 +66249,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdd84f29eebd450b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ed9a8b8bd5c48f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66787,7 +66788,7 @@
         <x:v>Administration</x:v>
       </x:c>
       <x:c r="C48" s="30" t="str">
-        <x:v>Only an ACTIVE SYSTEM_ADMIN may restore a PUBLISHING_SUSPENDED Club, and restoration requires one eligible current Club administrator.</x:v>
+        <x:v>Only an ACTIVE SYSTEM_ADMIN may restore a PUBLISHING_SUSPENDED Club. Restoration requires one eligible current Club administrator, which may be the reactivated original administrator; account reactivation alone never restores publishing.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="24" hidden="0" customHeight="1">
@@ -66804,7 +66805,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6632626804604ab8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5427e32a076d4334"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -67341,7 +67342,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R907b3f345dc74d88"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe82aaaaceeb4f50"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(admin): add account moderation and session revocation (#64) (#65)
</commit_message>
<xml_diff>
--- a/docs/requirements/UniConnect_Requirements_Baseline.xlsx
+++ b/docs/requirements/UniConnect_Requirements_Baseline.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="Rcf8013865f31425f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="R19e26ab60ec64ab8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="Rd5b7d80ce6234c46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="R5a8ebbee880d47d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="Rb897d9c835614911"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="R1031445abf4741f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="R3e3432dc7e4a4baa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Re41e933701ac4c6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="R91c5e0853a3f45fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="Rb590d7afb9534d5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="Rfaa9ca7984db4f97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="R86c04731cf3140f8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -929,7 +929,7 @@
         <x:color rgb="FF006100"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFC6EFCE"/>
         </x:patternFill>
       </x:fill>
@@ -940,7 +940,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -951,7 +951,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
@@ -33049,7 +33049,7 @@
 - ClubStatus becomes PUBLISHING_SUSPENDED and the reason/state change is audited.
 - New Club publications are blocked.
 - The Club profile and already-published announcements remain visible.
-- If suspension resulted from an unavailable administrator, publishing cannot be restored until an eligible replacement is appointed.</x:v>
+- If suspension resulted from an unavailable administrator, restoration requires exactly one eligible current CLUB_ADMINISTRATOR. Reactivating the original administrator may satisfy eligibility, but account reactivation does not restore publishing; an authorized SYSTEM_ADMIN must explicitly restore it under FR_83.</x:v>
       </x:c>
       <x:c r="K78" s="15" t="str">
         <x:v>High</x:v>
@@ -33599,7 +33599,8 @@
         <x:v>- Only an ACTIVE SYSTEM_ADMIN may restore publishing.
 - The Club currently has status PUBLISHING_SUSPENDED.
 - A reason or resolution note is required.
-- The Club has exactly one eligible current CLUB_ADMINISTRATOR.
+- The Club has exactly one eligible current CLUB_ADMINISTRATOR; this may be the original administrator after account reactivation.
+- Account reactivation never restores Club publishing; restoration is this explicit action.
 - ClubStatus becomes ACTIVE.
 - Authorized operators may publish again.
 - The state change is recorded in immutable audit history and produces one informational notification event.</x:v>
@@ -63492,9 +63493,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f06587077094fc5"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f1b418e25df4909"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc7e3952839a4826"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb249208ad2874dda"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -65770,7 +65771,7 @@
         <x:v>Called a Club an account and treated suspension as full invisibility.</x:v>
       </x:c>
       <x:c r="H78" s="31" t="str">
-        <x:v>Used canonical ClubStatus and limited suspension to new publishing.</x:v>
+        <x:v>Used canonical ClubStatus, limited suspension to new publishing, and clarified that a reactivated original administrator may satisfy eligibility while explicit FR_83 restoration remains required.</x:v>
       </x:c>
       <x:c r="I78" s="31" t="str">
         <x:v>UniConnect_Administration_Notification_Class_Diagram_Corrected.drawio</x:v>
@@ -66031,7 +66032,7 @@
         <x:v>Restoring Club publishing existed in the administration model but had no atomic functional requirement.</x:v>
       </x:c>
       <x:c r="H87" s="30" t="str">
-        <x:v>Added an authorized, audited restoration requirement with an eligible-administrator precondition.</x:v>
+        <x:v>Added an authorized, audited explicit restoration requirement; an eligible current administrator may be the reactivated original administrator, but reactivation alone never restores publishing.</x:v>
       </x:c>
       <x:c r="I87" s="30" t="str">
         <x:v>UniConnect_Administration_Notification_Class_Diagram_Corrected.drawio</x:v>
@@ -66248,7 +66249,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdd84f29eebd450b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ed9a8b8bd5c48f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66787,7 +66788,7 @@
         <x:v>Administration</x:v>
       </x:c>
       <x:c r="C48" s="30" t="str">
-        <x:v>Only an ACTIVE SYSTEM_ADMIN may restore a PUBLISHING_SUSPENDED Club, and restoration requires one eligible current Club administrator.</x:v>
+        <x:v>Only an ACTIVE SYSTEM_ADMIN may restore a PUBLISHING_SUSPENDED Club. Restoration requires one eligible current Club administrator, which may be the reactivated original administrator; account reactivation alone never restores publishing.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="24" hidden="0" customHeight="1">
@@ -66804,7 +66805,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6632626804604ab8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5427e32a076d4334"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -67341,7 +67342,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R907b3f345dc74d88"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe82aaaaceeb4f50"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(reporting): add content reports and moderation review (#71)
</commit_message>
<xml_diff>
--- a/docs/requirements/UniConnect_Requirements_Baseline.xlsx
+++ b/docs/requirements/UniConnect_Requirements_Baseline.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="R3e3432dc7e4a4baa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Re41e933701ac4c6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="R91c5e0853a3f45fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="Rb590d7afb9534d5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="Rfaa9ca7984db4f97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="R86c04731cf3140f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="R69afee22b363497e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Rdd512aa099184a48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="R452a5338ad554aa2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="Re70a34437f6244e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="R51536b33cf5741b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="Rc2b91a1f0f8c4310"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -32841,35 +32841,40 @@
         <x:v>FR_67</x:v>
       </x:c>
       <x:c r="C75" s="13" t="str">
-        <x:v>The system shall allow a System Admin to view content submitted for moderation.</x:v>
+        <x:v>The system shall allow an authenticated ACTIVE, non-anonymized user to submit a report about an accessible supported target and allow SYSTEM_ADMINISTRATION reviewers to resolve it with retained evidence and reporter notification.</x:v>
       </x:c>
       <x:c r="D75" s="12" t="str">
         <x:v>US_67</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
-        <x:v>Review Reported Content</x:v>
+        <x:v>Submit and Review a Content Report</x:v>
       </x:c>
       <x:c r="F75" s="19" t="str">
-        <x:v>System Admin</x:v>
+        <x:v>Authenticated member / System Administrator</x:v>
       </x:c>
       <x:c r="G75" s="19" t="str">
-        <x:v>to view reported content</x:v>
+        <x:v>to submit or review an accessible content report through its lifecycle</x:v>
       </x:c>
       <x:c r="H75" s="19" t="str">
-        <x:v>I can review the flagged contents before taking action.</x:v>
+        <x:v>reported content can be reviewed consistently while history and privacy are preserved.</x:v>
       </x:c>
       <x:c r="I75" s="13" t="str">
-        <x:v>As a System Admin, I want to view reported content, so that I can review the flagged contents before taking action.</x:v>
+        <x:v>As an authenticated member, I want to report accessible content and receive a resolution summary; as a System Administrator, I want to review the retained evidence and resolve the report consistently.</x:v>
       </x:c>
       <x:c r="J75" s="13" t="str">
-        <x:v>- Reports appear in a moderation queue.
-- Original content is displayed.
-- Report reason is displayed.
-- Content owner is identified.
-- Reports can be filtered by status.</x:v>
+        <x:v>- Any authenticated ACTIVE, non-anonymized user may submit regardless of selected context.
+- Supported targets are USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE; projects and career posts remain deferred until their modules exist.
+- The reporter must be able to access the target; inaccessible and nonexistent targets both return 404.
+- Minimal immutable evidence is captured through the owning module and is never returned in reporter DTOs.
+- One open report is allowed per reporter and target; different reporters remain independent and a later report is allowed after closure.
+- Lifecycle is SUBMITTED → UNDER_REVIEW → ACTION_TAKEN or NO_ACTION.
+- The first SYSTEM_ADMINISTRATION reviewer owns resolution; concurrent claims and decisions cannot overwrite each other.
+- Both outcomes require a reporter-visible resolution summary; internal notes and action details remain administrator-only.
+- Resolution, transition audit, optional action link, and one REPORT_RESOLVED notification commit atomically.
+- Identical retries create no duplicate audit or notification; conflicting terminal outcomes return 409.</x:v>
       </x:c>
       <x:c r="K75" s="15" t="str">
-        <x:v>Low</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="L75" s="15" t="str">
         <x:v>To Do</x:v>
@@ -32901,35 +32906,38 @@
         <x:v>FR_68</x:v>
       </x:c>
       <x:c r="C76" s="13" t="str">
-        <x:v>The system shall allow an ACTIVE SYSTEM_ADMIN to remove a reported Announcement, Project, JobPost, or Club that violates platform rules.</x:v>
+        <x:v>The system shall allow the reviewing ACTIVE SYSTEM_ADMIN to resolve a report as ACTION_TAKEN only by linking an already committed qualifying action verified through its owning module.</x:v>
       </x:c>
       <x:c r="D76" s="12" t="str">
         <x:v>US_68</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
-        <x:v>Remove Content That Violates Platform Rules</x:v>
+        <x:v>Resolve a Report with Verified Action Evidence</x:v>
       </x:c>
       <x:c r="F76" s="19" t="str">
-        <x:v>System Admin</x:v>
+        <x:v>Reviewing System Administrator</x:v>
       </x:c>
       <x:c r="G76" s="19" t="str">
-        <x:v>remove offending contents</x:v>
+        <x:v>to link a qualifying committed action when resolving a report</x:v>
       </x:c>
       <x:c r="H76" s="19" t="str">
-        <x:v>I can maintain a safe and professional environment for all users.</x:v>
+        <x:v>the report records what addressed it without granting or repeating moderation permissions.</x:v>
       </x:c>
       <x:c r="I76" s="13" t="str">
-        <x:v>As a System Admin, I want to remove offending contents, so that I can maintain a safe and professional environment for all users.</x:v>
+        <x:v>As the reviewing System Administrator, I want to link a verified action already committed through its owning module, so that the report records its outcome without executing another moderation action.</x:v>
       </x:c>
       <x:c r="J76" s="13" t="str">
-        <x:v>- Only an ACTIVE SYSTEM_ADMIN may remove a supported typed target.
-- A moderation reason is required.
-- The target changes to its REMOVED lifecycle state and is no longer publicly accessible.
-- The related report is resolved once the report model is defined.
-- A typed ModerationAction and immutable AuditLog record the administrator, target, previous/new state, reason, and timestamp.</x:v>
+        <x:v>- Resolution never executes a moderation action and never infers evidence from current target status.
+- USER accepts suspension of that account.
+- CLUB accepts publishing suspension or removal of that club.
+- ANNOUNCEMENT and EVENT accept removal by an existing authorized club operator, suspension of the captured author, or publishing suspension/removal of the captured parent club.
+- CHAT_MESSAGE accepts suspension of the captured sender.
+- Server-side checks verify the retained audit, target/author/club relationship, and that the action was not already reversed at resolution time.
+- Existing permissions for account, club, and publication actions remain unchanged; no administrative chat hiding, warning, or new publication-removal permission is created.
+- Historical action identity remains linked if the action is reversed later.</x:v>
       </x:c>
       <x:c r="K76" s="15" t="str">
-        <x:v>Low</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="L76" s="15" t="str">
         <x:v>To Do</x:v>
@@ -63493,9 +63501,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f1b418e25df4909"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f53d800d3e64eeb"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb249208ad2874dda"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dee722995414b4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -65678,16 +65686,16 @@
         <x:v>Administration &amp; Moderation</x:v>
       </x:c>
       <x:c r="F75" s="31" t="str">
-        <x:v>Deferred</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="G75" s="31" t="str">
-        <x:v>Content reporting still needs ContentReport, ReportStatus, submission, target, lifecycle, and resolution decisions.</x:v>
+        <x:v>Content reporting previously lacked approved target, access, lifecycle, concurrency, evidence, privacy, and notification rules.</x:v>
       </x:c>
       <x:c r="H75" s="31" t="str">
-        <x:v>Retained for long-term traceability but deferred from the one-month rebuild until its business rules and model are approved.</x:v>
+        <x:v>Approved the bounded USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE reporting lifecycle with owner-only reporter reads and SYSTEM_ADMINISTRATION review.</x:v>
       </x:c>
       <x:c r="I75" s="31" t="str">
-        <x:v>UniConnect_Administration_Notification_Class_Diagram_Corrected.drawio</x:v>
+        <x:v>Administration_Notification.drawio; One_to_One_Chat.drawio; CONTENT_REPORTING.md</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -65710,13 +65718,13 @@
         <x:v>Reworded</x:v>
       </x:c>
       <x:c r="G76" s="31" t="str">
-        <x:v>Used an untyped generic content target and physical-deletion language.</x:v>
+        <x:v>The prior wording granted generic SYSTEM_ADMIN content-removal authority and referenced unavailable Project and JobPost modules.</x:v>
       </x:c>
       <x:c r="H76" s="31" t="str">
-        <x:v>Aligned moderation removal with typed targets and retained lifecycle/audit records.</x:v>
+        <x:v>Separated report resolution from action execution, retained existing action permissions, and required a verified link to qualifying committed evidence.</x:v>
       </x:c>
       <x:c r="I76" s="31" t="str">
-        <x:v>UniConnect_Administration_Notification_Class_Diagram_Corrected.drawio</x:v>
+        <x:v>Administration_Notification.drawio; CONTENT_REPORTING.md</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -66249,7 +66257,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ed9a8b8bd5c48f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0eae1a1dbbc4ba0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66802,10 +66810,109 @@
         <x:v>Account anonymization is terminal: sessions and credentials are invalidated, identifiers are removed, and required historical records remain with anonymized attribution.</x:v>
       </x:c>
     </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="30" t="str">
+        <x:v>RP-01</x:v>
+      </x:c>
+      <x:c r="B50" s="30" t="str">
+        <x:v>Reporting</x:v>
+      </x:c>
+      <x:c r="C50" s="30" t="str">
+        <x:v>Any authenticated ACTIVE, non-anonymized user may submit a report regardless of selected context, but the target must be accessible through its owning module.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="30" t="str">
+        <x:v>RP-02</x:v>
+      </x:c>
+      <x:c r="B51" s="30" t="str">
+        <x:v>Reporting</x:v>
+      </x:c>
+      <x:c r="C51" s="30" t="str">
+        <x:v>Supported targets are USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE. Project and career-post targets remain deferred until their modules exist.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="30" t="str">
+        <x:v>RP-03</x:v>
+      </x:c>
+      <x:c r="B52" s="30" t="str">
+        <x:v>Reporting</x:v>
+      </x:c>
+      <x:c r="C52" s="30" t="str">
+        <x:v>The lifecycle is SUBMITTED to UNDER_REVIEW to ACTION_TAKEN or NO_ACTION. The first reviewer owns resolution, and concurrent transitions cannot overwrite a decision.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="30" t="str">
+        <x:v>RP-04</x:v>
+      </x:c>
+      <x:c r="B53" s="30" t="str">
+        <x:v>Reporting</x:v>
+      </x:c>
+      <x:c r="C53" s="30" t="str">
+        <x:v>One open report is allowed per reporter and target. Different reporters are independent, and a later report is allowed after the prior report closes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="30" t="str">
+        <x:v>RP-05</x:v>
+      </x:c>
+      <x:c r="B54" s="30" t="str">
+        <x:v>Reporting</x:v>
+      </x:c>
+      <x:c r="C54" s="30" t="str">
+        <x:v>ACTION_TAKEN links an already committed qualifying action verified through the owning module; resolving a report never executes moderation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="30" t="str">
+        <x:v>RP-06</x:v>
+      </x:c>
+      <x:c r="B55" s="30" t="str">
+        <x:v>Reporting</x:v>
+      </x:c>
+      <x:c r="C55" s="30" t="str">
+        <x:v>Reporter DTOs are owner-only and omit immutable snapshots, internal notes, action evidence, and audit history. Inaccessible and nonexistent targets both return 404.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="30" t="str">
+        <x:v>RP-07</x:v>
+      </x:c>
+      <x:c r="B56" s="30" t="str">
+        <x:v>Reporting</x:v>
+      </x:c>
+      <x:c r="C56" s="30" t="str">
+        <x:v>Terminal resolution, transition audit, optional action link, and one REPORT_RESOLVED notification commit atomically; identical retries are no-ops.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="30" t="str">
+        <x:v>RP-08</x:v>
+      </x:c>
+      <x:c r="B57" s="30" t="str">
+        <x:v>Reporting</x:v>
+      </x:c>
+      <x:c r="C57" s="30" t="str">
+        <x:v>Delete-for-everyone message text may be retained only as administrator evidence; delete-for-self messages remain inaccessible for new reports.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="30" t="str">
+        <x:v>RP-09</x:v>
+      </x:c>
+      <x:c r="B58" s="30" t="str">
+        <x:v>Reporting</x:v>
+      </x:c>
+      <x:c r="C58" s="30" t="str">
+        <x:v>Warnings, administrative chat hiding, and new publication-removal permissions are outside the bounded reporting phase.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5427e32a076d4334"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc76e8da9183d48ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66870,7 +66977,7 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="D5" s="115" t="str">
-        <x:v>The baseline now contains explicit announcement draft, publication, unpublishing and expiry behavior; a separate Event lifecycle; terminal account anonymization; and restoration of Club publishing. The one-month Implementation Scope prioritizes Authentication/Profile, Clubs, Connections/User Discovery, Announcements/Events, and One-to-One Chat as MUST. Project Teammate Finder is SHOULD. Content reporting and warnings remain traceable but are deliberately deferred until their rules and model are approved.</x:v>
+        <x:v>The baseline now contains explicit announcement draft, publication, unpublishing and expiry behavior; a separate Event lifecycle; terminal account anonymization; restoration of Club publishing; and the approved bounded content-reporting lifecycle. Warnings and unavailable project/career report targets remain deferred until their owning policies and modules are approved.</x:v>
       </x:c>
       <x:c r="E5" s="116"/>
       <x:c r="F5" s="116"/>
@@ -66939,12 +67046,12 @@
       </x:c>
       <x:c r="B10" t="n">
         <x:f>COUNTIF('Consistency Audit'!$F$2:$F$94,"Deferred")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="125" t="str">
-        <x:v>Deferred design decisions (outside the one-month rebuild scope)</x:v>
+        <x:v>Approved reporting decision</x:v>
       </x:c>
       <x:c r="B11" s="125"/>
       <x:c r="C11" s="125"/>
@@ -66956,10 +67063,10 @@
     </x:row>
     <x:row r="12" ht="52" customHeight="1">
       <x:c r="A12" s="128" t="str">
-        <x:v>FR_67 — Content reporting</x:v>
+        <x:v>FR_67–FR_68 — Content reporting</x:v>
       </x:c>
       <x:c r="B12" s="130" t="str">
-        <x:v>ContentReport, ReportStatus, ReportingService, report submission/target/lifecycle and resolution rules will be designed later. FR_67 remains in the long-term baseline and is DEFERRED for the one-month rebuild.</x:v>
+        <x:v>Approved bounded backend reporting for USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE with retained evidence, reviewer ownership, verified action links, reporter resolution notification, atomic history, and no action execution during resolution.</x:v>
       </x:c>
       <x:c r="C12" s="130"/>
       <x:c r="D12" s="130"/>
@@ -66973,7 +67080,7 @@
         <x:v>FR_69 — Warning system</x:v>
       </x:c>
       <x:c r="B13" s="130" t="str">
-        <x:v>issueWarning() and warning-related action, notification and audit types will be designed later. FR_69 remains in the long-term baseline and is DEFERRED for the one-month rebuild.</x:v>
+        <x:v>issueWarning() and warning-related action, notification, and audit types remain deferred until warning policy and model are approved.</x:v>
       </x:c>
       <x:c r="C13" s="130"/>
       <x:c r="D13" s="130"/>
@@ -67034,7 +67141,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="131" t="str">
-        <x:v>Reporting and warning design explicitly deferred without deleting FR_67 or FR_69</x:v>
+        <x:v>Reporting design approved for the bounded backend phase; warnings remain explicitly deferred</x:v>
       </x:c>
       <x:c r="B19" s="131"/>
       <x:c r="C19" s="131"/>
@@ -67271,7 +67378,7 @@
         <x:v>Account/Club moderation, anonymization and publishing restoration</x:v>
       </x:c>
       <x:c r="E13" s="30" t="str">
-        <x:v>Reporting and warnings are excluded from this scope.</x:v>
+        <x:v>Existing account, Club, and publication actions remain authoritative; report resolution may verify their audits but never executes them.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="48" customHeight="1">
@@ -67308,21 +67415,38 @@
         <x:v>Retained in the product baseline for later implementation.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="48" customHeight="1">
+    <x:row r="16" ht="36" hidden="0" customHeight="1">
       <x:c r="A16" s="30" t="str">
-        <x:v>Content Reporting &amp; Warning System</x:v>
+        <x:v>Content Reporting</x:v>
       </x:c>
       <x:c r="B16" s="30" t="str">
+        <x:v>SHOULD</x:v>
+      </x:c>
+      <x:c r="C16" s="30" t="str">
+        <x:v>FR_67–FR_68</x:v>
+      </x:c>
+      <x:c r="D16" s="30" t="str">
+        <x:v>Backend submission, retained evidence, administration review, verified action linking, audit, and resolution notification</x:v>
+      </x:c>
+      <x:c r="E16" s="30" t="str">
+        <x:v>Targets are USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE. Flutter screens and unavailable project/career targets remain separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="24" hidden="0" customHeight="1">
+      <x:c r="A17" s="30" t="str">
+        <x:v>Warning System</x:v>
+      </x:c>
+      <x:c r="B17" s="30" t="str">
         <x:v>DEFERRED</x:v>
       </x:c>
-      <x:c r="C16" s="30" t="str">
-        <x:v>FR_67, FR_69</x:v>
-      </x:c>
-      <x:c r="D16" s="30" t="str">
-        <x:v>No implementation until rules and model are approved</x:v>
-      </x:c>
-      <x:c r="E16" s="30" t="str">
-        <x:v>ContentReport, ReportStatus, ReportingService, issueWarning(), and warning action/notification/audit types will be designed later.</x:v>
+      <x:c r="C17" s="30" t="str">
+        <x:v>FR_69</x:v>
+      </x:c>
+      <x:c r="D17" s="30" t="str">
+        <x:v>No implementation until warning policy and model are approved</x:v>
+      </x:c>
+      <x:c r="E17" s="30" t="str">
+        <x:v>Warning action, notification, audit, and member-history rules remain deferred.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -67342,7 +67466,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe82aaaaceeb4f50"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c17866468044af1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(reporting): implement content reports and review (#71) (#72)
* feat(reporting): add content reports and moderation review (#71)

* style(frontend): format notification page and tests
</commit_message>
<xml_diff>
--- a/docs/requirements/UniConnect_Requirements_Baseline.xlsx
+++ b/docs/requirements/UniConnect_Requirements_Baseline.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="R3e3432dc7e4a4baa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Re41e933701ac4c6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="R91c5e0853a3f45fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="Rb590d7afb9534d5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="Rfaa9ca7984db4f97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="R86c04731cf3140f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="R69afee22b363497e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Rdd512aa099184a48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="R452a5338ad554aa2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="Re70a34437f6244e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="R51536b33cf5741b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="Rc2b91a1f0f8c4310"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -32841,35 +32841,40 @@
         <x:v>FR_67</x:v>
       </x:c>
       <x:c r="C75" s="13" t="str">
-        <x:v>The system shall allow a System Admin to view content submitted for moderation.</x:v>
+        <x:v>The system shall allow an authenticated ACTIVE, non-anonymized user to submit a report about an accessible supported target and allow SYSTEM_ADMINISTRATION reviewers to resolve it with retained evidence and reporter notification.</x:v>
       </x:c>
       <x:c r="D75" s="12" t="str">
         <x:v>US_67</x:v>
       </x:c>
       <x:c r="E75" s="14" t="str">
-        <x:v>Review Reported Content</x:v>
+        <x:v>Submit and Review a Content Report</x:v>
       </x:c>
       <x:c r="F75" s="19" t="str">
-        <x:v>System Admin</x:v>
+        <x:v>Authenticated member / System Administrator</x:v>
       </x:c>
       <x:c r="G75" s="19" t="str">
-        <x:v>to view reported content</x:v>
+        <x:v>to submit or review an accessible content report through its lifecycle</x:v>
       </x:c>
       <x:c r="H75" s="19" t="str">
-        <x:v>I can review the flagged contents before taking action.</x:v>
+        <x:v>reported content can be reviewed consistently while history and privacy are preserved.</x:v>
       </x:c>
       <x:c r="I75" s="13" t="str">
-        <x:v>As a System Admin, I want to view reported content, so that I can review the flagged contents before taking action.</x:v>
+        <x:v>As an authenticated member, I want to report accessible content and receive a resolution summary; as a System Administrator, I want to review the retained evidence and resolve the report consistently.</x:v>
       </x:c>
       <x:c r="J75" s="13" t="str">
-        <x:v>- Reports appear in a moderation queue.
-- Original content is displayed.
-- Report reason is displayed.
-- Content owner is identified.
-- Reports can be filtered by status.</x:v>
+        <x:v>- Any authenticated ACTIVE, non-anonymized user may submit regardless of selected context.
+- Supported targets are USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE; projects and career posts remain deferred until their modules exist.
+- The reporter must be able to access the target; inaccessible and nonexistent targets both return 404.
+- Minimal immutable evidence is captured through the owning module and is never returned in reporter DTOs.
+- One open report is allowed per reporter and target; different reporters remain independent and a later report is allowed after closure.
+- Lifecycle is SUBMITTED → UNDER_REVIEW → ACTION_TAKEN or NO_ACTION.
+- The first SYSTEM_ADMINISTRATION reviewer owns resolution; concurrent claims and decisions cannot overwrite each other.
+- Both outcomes require a reporter-visible resolution summary; internal notes and action details remain administrator-only.
+- Resolution, transition audit, optional action link, and one REPORT_RESOLVED notification commit atomically.
+- Identical retries create no duplicate audit or notification; conflicting terminal outcomes return 409.</x:v>
       </x:c>
       <x:c r="K75" s="15" t="str">
-        <x:v>Low</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="L75" s="15" t="str">
         <x:v>To Do</x:v>
@@ -32901,35 +32906,38 @@
         <x:v>FR_68</x:v>
       </x:c>
       <x:c r="C76" s="13" t="str">
-        <x:v>The system shall allow an ACTIVE SYSTEM_ADMIN to remove a reported Announcement, Project, JobPost, or Club that violates platform rules.</x:v>
+        <x:v>The system shall allow the reviewing ACTIVE SYSTEM_ADMIN to resolve a report as ACTION_TAKEN only by linking an already committed qualifying action verified through its owning module.</x:v>
       </x:c>
       <x:c r="D76" s="12" t="str">
         <x:v>US_68</x:v>
       </x:c>
       <x:c r="E76" s="14" t="str">
-        <x:v>Remove Content That Violates Platform Rules</x:v>
+        <x:v>Resolve a Report with Verified Action Evidence</x:v>
       </x:c>
       <x:c r="F76" s="19" t="str">
-        <x:v>System Admin</x:v>
+        <x:v>Reviewing System Administrator</x:v>
       </x:c>
       <x:c r="G76" s="19" t="str">
-        <x:v>remove offending contents</x:v>
+        <x:v>to link a qualifying committed action when resolving a report</x:v>
       </x:c>
       <x:c r="H76" s="19" t="str">
-        <x:v>I can maintain a safe and professional environment for all users.</x:v>
+        <x:v>the report records what addressed it without granting or repeating moderation permissions.</x:v>
       </x:c>
       <x:c r="I76" s="13" t="str">
-        <x:v>As a System Admin, I want to remove offending contents, so that I can maintain a safe and professional environment for all users.</x:v>
+        <x:v>As the reviewing System Administrator, I want to link a verified action already committed through its owning module, so that the report records its outcome without executing another moderation action.</x:v>
       </x:c>
       <x:c r="J76" s="13" t="str">
-        <x:v>- Only an ACTIVE SYSTEM_ADMIN may remove a supported typed target.
-- A moderation reason is required.
-- The target changes to its REMOVED lifecycle state and is no longer publicly accessible.
-- The related report is resolved once the report model is defined.
-- A typed ModerationAction and immutable AuditLog record the administrator, target, previous/new state, reason, and timestamp.</x:v>
+        <x:v>- Resolution never executes a moderation action and never infers evidence from current target status.
+- USER accepts suspension of that account.
+- CLUB accepts publishing suspension or removal of that club.
+- ANNOUNCEMENT and EVENT accept removal by an existing authorized club operator, suspension of the captured author, or publishing suspension/removal of the captured parent club.
+- CHAT_MESSAGE accepts suspension of the captured sender.
+- Server-side checks verify the retained audit, target/author/club relationship, and that the action was not already reversed at resolution time.
+- Existing permissions for account, club, and publication actions remain unchanged; no administrative chat hiding, warning, or new publication-removal permission is created.
+- Historical action identity remains linked if the action is reversed later.</x:v>
       </x:c>
       <x:c r="K76" s="15" t="str">
-        <x:v>Low</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="L76" s="15" t="str">
         <x:v>To Do</x:v>
@@ -63493,9 +63501,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f1b418e25df4909"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f53d800d3e64eeb"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb249208ad2874dda"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dee722995414b4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -65678,16 +65686,16 @@
         <x:v>Administration &amp; Moderation</x:v>
       </x:c>
       <x:c r="F75" s="31" t="str">
-        <x:v>Deferred</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="G75" s="31" t="str">
-        <x:v>Content reporting still needs ContentReport, ReportStatus, submission, target, lifecycle, and resolution decisions.</x:v>
+        <x:v>Content reporting previously lacked approved target, access, lifecycle, concurrency, evidence, privacy, and notification rules.</x:v>
       </x:c>
       <x:c r="H75" s="31" t="str">
-        <x:v>Retained for long-term traceability but deferred from the one-month rebuild until its business rules and model are approved.</x:v>
+        <x:v>Approved the bounded USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE reporting lifecycle with owner-only reporter reads and SYSTEM_ADMINISTRATION review.</x:v>
       </x:c>
       <x:c r="I75" s="31" t="str">
-        <x:v>UniConnect_Administration_Notification_Class_Diagram_Corrected.drawio</x:v>
+        <x:v>Administration_Notification.drawio; One_to_One_Chat.drawio; CONTENT_REPORTING.md</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -65710,13 +65718,13 @@
         <x:v>Reworded</x:v>
       </x:c>
       <x:c r="G76" s="31" t="str">
-        <x:v>Used an untyped generic content target and physical-deletion language.</x:v>
+        <x:v>The prior wording granted generic SYSTEM_ADMIN content-removal authority and referenced unavailable Project and JobPost modules.</x:v>
       </x:c>
       <x:c r="H76" s="31" t="str">
-        <x:v>Aligned moderation removal with typed targets and retained lifecycle/audit records.</x:v>
+        <x:v>Separated report resolution from action execution, retained existing action permissions, and required a verified link to qualifying committed evidence.</x:v>
       </x:c>
       <x:c r="I76" s="31" t="str">
-        <x:v>UniConnect_Administration_Notification_Class_Diagram_Corrected.drawio</x:v>
+        <x:v>Administration_Notification.drawio; CONTENT_REPORTING.md</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -66249,7 +66257,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ed9a8b8bd5c48f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0eae1a1dbbc4ba0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66802,10 +66810,109 @@
         <x:v>Account anonymization is terminal: sessions and credentials are invalidated, identifiers are removed, and required historical records remain with anonymized attribution.</x:v>
       </x:c>
     </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="30" t="str">
+        <x:v>RP-01</x:v>
+      </x:c>
+      <x:c r="B50" s="30" t="str">
+        <x:v>Reporting</x:v>
+      </x:c>
+      <x:c r="C50" s="30" t="str">
+        <x:v>Any authenticated ACTIVE, non-anonymized user may submit a report regardless of selected context, but the target must be accessible through its owning module.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="30" t="str">
+        <x:v>RP-02</x:v>
+      </x:c>
+      <x:c r="B51" s="30" t="str">
+        <x:v>Reporting</x:v>
+      </x:c>
+      <x:c r="C51" s="30" t="str">
+        <x:v>Supported targets are USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE. Project and career-post targets remain deferred until their modules exist.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="30" t="str">
+        <x:v>RP-03</x:v>
+      </x:c>
+      <x:c r="B52" s="30" t="str">
+        <x:v>Reporting</x:v>
+      </x:c>
+      <x:c r="C52" s="30" t="str">
+        <x:v>The lifecycle is SUBMITTED to UNDER_REVIEW to ACTION_TAKEN or NO_ACTION. The first reviewer owns resolution, and concurrent transitions cannot overwrite a decision.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="30" t="str">
+        <x:v>RP-04</x:v>
+      </x:c>
+      <x:c r="B53" s="30" t="str">
+        <x:v>Reporting</x:v>
+      </x:c>
+      <x:c r="C53" s="30" t="str">
+        <x:v>One open report is allowed per reporter and target. Different reporters are independent, and a later report is allowed after the prior report closes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="30" t="str">
+        <x:v>RP-05</x:v>
+      </x:c>
+      <x:c r="B54" s="30" t="str">
+        <x:v>Reporting</x:v>
+      </x:c>
+      <x:c r="C54" s="30" t="str">
+        <x:v>ACTION_TAKEN links an already committed qualifying action verified through the owning module; resolving a report never executes moderation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="30" t="str">
+        <x:v>RP-06</x:v>
+      </x:c>
+      <x:c r="B55" s="30" t="str">
+        <x:v>Reporting</x:v>
+      </x:c>
+      <x:c r="C55" s="30" t="str">
+        <x:v>Reporter DTOs are owner-only and omit immutable snapshots, internal notes, action evidence, and audit history. Inaccessible and nonexistent targets both return 404.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="30" t="str">
+        <x:v>RP-07</x:v>
+      </x:c>
+      <x:c r="B56" s="30" t="str">
+        <x:v>Reporting</x:v>
+      </x:c>
+      <x:c r="C56" s="30" t="str">
+        <x:v>Terminal resolution, transition audit, optional action link, and one REPORT_RESOLVED notification commit atomically; identical retries are no-ops.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="30" t="str">
+        <x:v>RP-08</x:v>
+      </x:c>
+      <x:c r="B57" s="30" t="str">
+        <x:v>Reporting</x:v>
+      </x:c>
+      <x:c r="C57" s="30" t="str">
+        <x:v>Delete-for-everyone message text may be retained only as administrator evidence; delete-for-self messages remain inaccessible for new reports.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="30" t="str">
+        <x:v>RP-09</x:v>
+      </x:c>
+      <x:c r="B58" s="30" t="str">
+        <x:v>Reporting</x:v>
+      </x:c>
+      <x:c r="C58" s="30" t="str">
+        <x:v>Warnings, administrative chat hiding, and new publication-removal permissions are outside the bounded reporting phase.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5427e32a076d4334"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc76e8da9183d48ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66870,7 +66977,7 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="D5" s="115" t="str">
-        <x:v>The baseline now contains explicit announcement draft, publication, unpublishing and expiry behavior; a separate Event lifecycle; terminal account anonymization; and restoration of Club publishing. The one-month Implementation Scope prioritizes Authentication/Profile, Clubs, Connections/User Discovery, Announcements/Events, and One-to-One Chat as MUST. Project Teammate Finder is SHOULD. Content reporting and warnings remain traceable but are deliberately deferred until their rules and model are approved.</x:v>
+        <x:v>The baseline now contains explicit announcement draft, publication, unpublishing and expiry behavior; a separate Event lifecycle; terminal account anonymization; restoration of Club publishing; and the approved bounded content-reporting lifecycle. Warnings and unavailable project/career report targets remain deferred until their owning policies and modules are approved.</x:v>
       </x:c>
       <x:c r="E5" s="116"/>
       <x:c r="F5" s="116"/>
@@ -66939,12 +67046,12 @@
       </x:c>
       <x:c r="B10" t="n">
         <x:f>COUNTIF('Consistency Audit'!$F$2:$F$94,"Deferred")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="125" t="str">
-        <x:v>Deferred design decisions (outside the one-month rebuild scope)</x:v>
+        <x:v>Approved reporting decision</x:v>
       </x:c>
       <x:c r="B11" s="125"/>
       <x:c r="C11" s="125"/>
@@ -66956,10 +67063,10 @@
     </x:row>
     <x:row r="12" ht="52" customHeight="1">
       <x:c r="A12" s="128" t="str">
-        <x:v>FR_67 — Content reporting</x:v>
+        <x:v>FR_67–FR_68 — Content reporting</x:v>
       </x:c>
       <x:c r="B12" s="130" t="str">
-        <x:v>ContentReport, ReportStatus, ReportingService, report submission/target/lifecycle and resolution rules will be designed later. FR_67 remains in the long-term baseline and is DEFERRED for the one-month rebuild.</x:v>
+        <x:v>Approved bounded backend reporting for USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE with retained evidence, reviewer ownership, verified action links, reporter resolution notification, atomic history, and no action execution during resolution.</x:v>
       </x:c>
       <x:c r="C12" s="130"/>
       <x:c r="D12" s="130"/>
@@ -66973,7 +67080,7 @@
         <x:v>FR_69 — Warning system</x:v>
       </x:c>
       <x:c r="B13" s="130" t="str">
-        <x:v>issueWarning() and warning-related action, notification and audit types will be designed later. FR_69 remains in the long-term baseline and is DEFERRED for the one-month rebuild.</x:v>
+        <x:v>issueWarning() and warning-related action, notification, and audit types remain deferred until warning policy and model are approved.</x:v>
       </x:c>
       <x:c r="C13" s="130"/>
       <x:c r="D13" s="130"/>
@@ -67034,7 +67141,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="131" t="str">
-        <x:v>Reporting and warning design explicitly deferred without deleting FR_67 or FR_69</x:v>
+        <x:v>Reporting design approved for the bounded backend phase; warnings remain explicitly deferred</x:v>
       </x:c>
       <x:c r="B19" s="131"/>
       <x:c r="C19" s="131"/>
@@ -67271,7 +67378,7 @@
         <x:v>Account/Club moderation, anonymization and publishing restoration</x:v>
       </x:c>
       <x:c r="E13" s="30" t="str">
-        <x:v>Reporting and warnings are excluded from this scope.</x:v>
+        <x:v>Existing account, Club, and publication actions remain authoritative; report resolution may verify their audits but never executes them.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="48" customHeight="1">
@@ -67308,21 +67415,38 @@
         <x:v>Retained in the product baseline for later implementation.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="48" customHeight="1">
+    <x:row r="16" ht="36" hidden="0" customHeight="1">
       <x:c r="A16" s="30" t="str">
-        <x:v>Content Reporting &amp; Warning System</x:v>
+        <x:v>Content Reporting</x:v>
       </x:c>
       <x:c r="B16" s="30" t="str">
+        <x:v>SHOULD</x:v>
+      </x:c>
+      <x:c r="C16" s="30" t="str">
+        <x:v>FR_67–FR_68</x:v>
+      </x:c>
+      <x:c r="D16" s="30" t="str">
+        <x:v>Backend submission, retained evidence, administration review, verified action linking, audit, and resolution notification</x:v>
+      </x:c>
+      <x:c r="E16" s="30" t="str">
+        <x:v>Targets are USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE. Flutter screens and unavailable project/career targets remain separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="24" hidden="0" customHeight="1">
+      <x:c r="A17" s="30" t="str">
+        <x:v>Warning System</x:v>
+      </x:c>
+      <x:c r="B17" s="30" t="str">
         <x:v>DEFERRED</x:v>
       </x:c>
-      <x:c r="C16" s="30" t="str">
-        <x:v>FR_67, FR_69</x:v>
-      </x:c>
-      <x:c r="D16" s="30" t="str">
-        <x:v>No implementation until rules and model are approved</x:v>
-      </x:c>
-      <x:c r="E16" s="30" t="str">
-        <x:v>ContentReport, ReportStatus, ReportingService, issueWarning(), and warning action/notification/audit types will be designed later.</x:v>
+      <x:c r="C17" s="30" t="str">
+        <x:v>FR_69</x:v>
+      </x:c>
+      <x:c r="D17" s="30" t="str">
+        <x:v>No implementation until warning policy and model are approved</x:v>
+      </x:c>
+      <x:c r="E17" s="30" t="str">
+        <x:v>Warning action, notification, audit, and member-history rules remain deferred.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -67342,7 +67466,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe82aaaaceeb4f50"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c17866468044af1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(project): add recruitment and team membership (#77)
</commit_message>
<xml_diff>
--- a/docs/requirements/UniConnect_Requirements_Baseline.xlsx
+++ b/docs/requirements/UniConnect_Requirements_Baseline.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="R69afee22b363497e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Rdd512aa099184a48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="R452a5338ad554aa2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="Re70a34437f6244e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="R51536b33cf5741b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="Rc2b91a1f0f8c4310"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="Rc05b016315274bf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Re2a21074ceed4a0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="R253303f188904593"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="R87d3e2b5a8454eba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="Rf4faa6cd2798456e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="Raa032e71943d4aac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -30450,7 +30450,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="L35" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>To Do</x:v>
       </x:c>
       <x:c r="M35" s="16"/>
       <x:c r="N35" s="16"/>
@@ -30509,7 +30509,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="L36" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>To Do</x:v>
       </x:c>
       <x:c r="M36" s="16"/>
       <x:c r="N36" s="16"/>
@@ -30570,7 +30570,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="L37" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>To Do</x:v>
       </x:c>
       <x:c r="M37" s="16"/>
       <x:c r="N37" s="16"/>
@@ -30591,7 +30591,7 @@
       <x:c r="AC37" s="16"/>
       <x:c r="AD37" s="16"/>
     </x:row>
-    <x:row r="38" ht="22.5" customHeight="1">
+    <x:row r="38" ht="156" hidden="0" customHeight="1">
       <x:c r="A38" s="11" t="n">
         <x:v>37</x:v>
       </x:c>
@@ -30620,17 +30620,18 @@
         <x:v>As a Student, I want to browse available project posts using filters and sorting options, so that I can find projects that match my skills and schedules efficiently.</x:v>
       </x:c>
       <x:c r="J38" s="13" t="str">
-        <x:v>- Open projects are displayed.
-- Skill, department, and status filters are available.
-- Sorting by date or deadline is available.
-- Project cards show key details.
-- Results are paginated.</x:v>
+        <x:v>- Default browse returns non-expired OPEN projects, including AVAILABLE and FULL projects.
+- Stored status and derived availability are separate filters and combine with AND.
+- Availability values are AVAILABLE, FULL, EXPIRED, and CLOSED.
+- Skill and creator-current-department filters are available.
+- Sorting supports newest-created and earliest-deadline order.
+- Results are paginated; DELETED projects never appear.</x:v>
       </x:c>
       <x:c r="K38" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L38" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M38" s="16"/>
       <x:c r="N38" s="16"/>
@@ -30651,7 +30652,7 @@
       <x:c r="AC38" s="16"/>
       <x:c r="AD38" s="16"/>
     </x:row>
-    <x:row r="39" ht="22.5" customHeight="1">
+    <x:row r="39" ht="132" hidden="0" customHeight="1">
       <x:c r="A39" s="11" t="n">
         <x:v>38</x:v>
       </x:c>
@@ -30680,17 +30681,17 @@
         <x:v>As a Student, I want to view the complete information of a selected project post, so that I can fully understand the project scope and requirements before deciding to join.</x:v>
       </x:c>
       <x:c r="J39" s="13" t="str">
-        <x:v>- Title and description are shown.
-- Required skills are shown.
-- Creator is shown.
-- Remaining positions are shown.
-- Current application status is shown.</x:v>
+        <x:v>- Title, description, skills, creator attribution, deadline, and lifecycle status are shown.
+- Membership count, vacancies, fullness, and availability are derived.
+- The current Student's lifetime application status is shown when one exists.
+- Closed and expired projects retain direct details.
+- DELETED projects return 404 from ordinary endpoints.</x:v>
       </x:c>
       <x:c r="K39" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L39" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M39" s="16"/>
       <x:c r="N39" s="16"/>
@@ -30711,7 +30712,7 @@
       <x:c r="AC39" s="16"/>
       <x:c r="AD39" s="16"/>
     </x:row>
-    <x:row r="40" ht="22.5" customHeight="1">
+    <x:row r="40" ht="156" hidden="0" customHeight="1">
       <x:c r="A40" s="11" t="n">
         <x:v>39</x:v>
       </x:c>
@@ -30740,18 +30741,18 @@
         <x:v>As a Student, I want to create a project post containing project details and required skills, so that I can attract suitable teammates who can contribute to my project.</x:v>
       </x:c>
       <x:c r="J40" s="13" t="str">
-        <x:v>- Title and description are required.
-- At least one required skill is selected.
-- teamSizeLimit is total capacity including the creator and is at least 2.
-- The Project is created with ProjectStatus = OPEN.
-- Creation atomically creates the sole CREATOR ProjectMembership.
-- openPositionCount is calculated from teamSizeLimit minus current memberships.</x:v>
+        <x:v>- Only an ACTIVE, non-anonymized STUDENT may create.
+- Title, description, applicationDeadline, and at least one required skill are required.
+- teamSizeLimit is total capacity including the creator and is between 2 and 100.
+- The deadline is valid through that date in Asia/Dhaka.
+- ProjectStatus is OPEN and the sole CREATOR membership is created atomically.
+- Membership count, vacancies, fullness, expiry, and availability are derived rather than stored.</x:v>
       </x:c>
       <x:c r="K40" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L40" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M40" s="16"/>
       <x:c r="N40" s="16"/>
@@ -30772,7 +30773,7 @@
       <x:c r="AC40" s="16"/>
       <x:c r="AD40" s="16"/>
     </x:row>
-    <x:row r="41" ht="22.5" customHeight="1">
+    <x:row r="41" ht="180" hidden="0" customHeight="1">
       <x:c r="A41" s="11" t="n">
         <x:v>40</x:v>
       </x:c>
@@ -30801,18 +30802,18 @@
         <x:v>As an eligible Student, I want to apply to an open project, so that I can join projects that interest me and fit my skills.</x:v>
       </x:c>
       <x:c r="J41" s="13" t="str">
-        <x:v>- The applicant has PlatformRole = STUDENT and AccountStatus = ACTIVE.
-- The Project is OPEN and has not been soft-deleted.
-- The creator and existing members cannot apply.
-- At most one application exists for the project/applicant pair.
-- The optional message is limited to 500 characters.
-- A valid application is stored as PENDING.</x:v>
+        <x:v>- Applicant and creator are currently ACTIVE, non-anonymized STUDENT accounts.
+- Project is OPEN, non-expired, not DELETED, and has a vacancy.
+- Creator and existing members cannot apply.
+- Exactly one lifetime application exists per project/applicant pair; withdrawal and reapplication are unavailable.
+- Optional message is at most 500 characters.
+- A valid application is stored as PENDING; the creator receives no application-received notification.</x:v>
       </x:c>
       <x:c r="K41" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L41" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M41" s="16"/>
       <x:c r="N41" s="16"/>
@@ -30833,7 +30834,7 @@
       <x:c r="AC41" s="16"/>
       <x:c r="AD41" s="16"/>
     </x:row>
-    <x:row r="42" ht="22.5" customHeight="1">
+    <x:row r="42" ht="96" hidden="0" customHeight="1">
       <x:c r="A42" s="11" t="n">
         <x:v>41</x:v>
       </x:c>
@@ -30862,17 +30863,16 @@
         <x:v>As the creator of a project, I want to view applications submitted to that project, so that I can review interested students and evaluate their suitability.</x:v>
       </x:c>
       <x:c r="J42" s="13" t="str">
-        <x:v>- Only the creator can view applications.
-- Application status is visible.
-- Applicant profile summary is shown.
-- Applicant message is shown.
-- Applications can be ordered by time.</x:v>
+        <x:v>- Only the ACTIVE creator may view applications.
+- Pending applications remain visible and reviewable after closing or expiry.
+- Applicant attribution, message, status, and UTC lifecycle timestamps are shown.
+- Deleted projects return 404 from ordinary endpoints.</x:v>
       </x:c>
       <x:c r="K42" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L42" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M42" s="16"/>
       <x:c r="N42" s="16"/>
@@ -30893,7 +30893,7 @@
       <x:c r="AC42" s="16"/>
       <x:c r="AD42" s="16"/>
     </x:row>
-    <x:row r="43" ht="22.5" customHeight="1">
+    <x:row r="43" ht="180" hidden="0" customHeight="1">
       <x:c r="A43" s="11" t="n">
         <x:v>42</x:v>
       </x:c>
@@ -30922,18 +30922,18 @@
         <x:v>As the creator of a project, I want to accept suitable applicants and decline unsuitable ones, so that I can select the best candidates for my team.</x:v>
       </x:c>
       <x:c r="J43" s="13" t="str">
-        <x:v>- Only the Project's creator may process an application.
-- Only PENDING applications may transition to ACCEPTED or REJECTED.
-- Acceptance atomically rechecks capacity, changes the application to ACCEPTED, and creates one TEAMMATE ProjectMembership.
-- Acceptance fails without partial change when capacity is full.
-- Rejection changes the application to REJECTED without creating membership.
-- The applicant receives one decision notification.</x:v>
+        <x:v>- Only the ACTIVE creator may process an application.
+- Only PENDING transitions to ACCEPTED or REJECTED; identical retries return the existing result.
+- Acceptance atomically locks, rechecks applicant eligibility and capacity, creates one TEAMMATE membership, audits, and notifies.
+- Capacity cannot be exceeded and partial acceptance cannot commit.
+- Rejection audits and notifies without membership.
+- Conflicting terminal retries return 409; identical retries duplicate nothing.</x:v>
       </x:c>
       <x:c r="K43" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L43" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M43" s="16"/>
       <x:c r="N43" s="16"/>
@@ -30954,7 +30954,7 @@
       <x:c r="AC43" s="16"/>
       <x:c r="AD43" s="16"/>
     </x:row>
-    <x:row r="44" ht="22.5" customHeight="1">
+    <x:row r="44" ht="108" hidden="0" customHeight="1">
       <x:c r="A44" s="11" t="n">
         <x:v>43</x:v>
       </x:c>
@@ -30983,17 +30983,17 @@
         <x:v>As the creator of a project, I want to update the project post, so that I can keep project details accurate and relevant for the future applicants.</x:v>
       </x:c>
       <x:c r="J44" s="13" t="str">
-        <x:v>- Only creator can edit.
-- Current values are shown.
-- Required fields cannot be removed.
-- Invalid values are rejected.
-- Valid changes appear immediately.</x:v>
+        <x:v>- Only the ACTIVE creator may edit a non-deleted OPEN or CLOSED Project.
+- Required fields remain valid and at least one skill remains required.
+- teamSizeLimit cannot be reduced below current membership.
+- Lifecycle timestamps are UTC.
+- Extending an OPEN Project's deadline can restore application availability.</x:v>
       </x:c>
       <x:c r="K44" s="15" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="L44" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M44" s="16"/>
       <x:c r="N44" s="16"/>
@@ -31014,7 +31014,7 @@
       <x:c r="AC44" s="16"/>
       <x:c r="AD44" s="16"/>
     </x:row>
-    <x:row r="45" ht="22.5" customHeight="1">
+    <x:row r="45" ht="132" hidden="0" customHeight="1">
       <x:c r="A45" s="11" t="n">
         <x:v>44</x:v>
       </x:c>
@@ -31043,18 +31043,17 @@
         <x:v>As a Project Creator whose available positions are filled, I want to close recruitment so that students do not spend time applying to an unavailable project.</x:v>
       </x:c>
       <x:c r="J45" s="13" t="str">
-        <x:v>- Only the creator may close an OPEN Project.
-- Closing changes ProjectStatus to CLOSED and rejects new applications.
-- Applications submitted before closing remain reviewable.
-- A pending pre-closing application may be accepted only while capacity remains.
-- The Project remains visible unless separately soft-deleted.
-- Closed recruitment is clearly displayed.</x:v>
+        <x:v>- Only the ACTIVE creator may close a non-deleted Project.
+- Closing is idempotent, sets ProjectStatus = CLOSED, records closedAt in UTC, and blocks new applications.
+- Pending pre-closing applications remain reviewable after close or expiry.
+- Acceptance remains possible only while capacity and applicant eligibility permit.
+- Closed projects retain direct details and explicit status/availability-filter browsing.</x:v>
       </x:c>
       <x:c r="K45" s="15" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="L45" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M45" s="16"/>
       <x:c r="N45" s="16"/>
@@ -31075,7 +31074,7 @@
       <x:c r="AC45" s="16"/>
       <x:c r="AD45" s="16"/>
     </x:row>
-    <x:row r="46" ht="22.5" customHeight="1">
+    <x:row r="46" ht="108" hidden="0" customHeight="1">
       <x:c r="A46" s="11" t="n">
         <x:v>45</x:v>
       </x:c>
@@ -31104,17 +31103,16 @@
         <x:v>As a Project Creator whose team has gained another vacancy, I want to reopen recruitment so that new candidates can apply.</x:v>
       </x:c>
       <x:c r="J46" s="13" t="str">
-        <x:v>- Only the creator may reopen the Project.
-- The Project is CLOSED, not DELETED, and has at least one derived open position.
-- Reopening changes ProjectStatus to OPEN.
-- New applications are accepted after reopening.
-- The Project returns to open-project browse results.</x:v>
+        <x:v>- Only the ACTIVE creator may reopen.
+- Project is CLOSED, non-deleted, has at least one vacancy, and has a deadline valid today or later in Asia/Dhaka.
+- Reopening changes ProjectStatus to OPEN and clears closedAt.
+- New applications become available only while the project remains non-expired and not full.</x:v>
       </x:c>
       <x:c r="K46" s="15" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="L46" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M46" s="16"/>
       <x:c r="N46" s="16"/>
@@ -31135,7 +31133,7 @@
       <x:c r="AC46" s="16"/>
       <x:c r="AD46" s="16"/>
     </x:row>
-    <x:row r="47" ht="22.5" customHeight="1">
+    <x:row r="47" ht="168" hidden="0" customHeight="1">
       <x:c r="A47" s="11" t="n">
         <x:v>46</x:v>
       </x:c>
@@ -31164,18 +31162,18 @@
         <x:v>As the creator of a Project, I want to remove it from normal use after confirmation so that outdated or abandoned projects no longer appear while historical records are preserved.</x:v>
       </x:c>
       <x:c r="J47" s="13" t="str">
-        <x:v>- Only the creator may initiate deletion.
-- Explicit confirmation is required; cancelling leaves the Project unchanged.
-- Confirmation sets ProjectStatus = DELETED and deletedAt.
-- The Project disappears from normal browse and search.
-- Project, application, membership, and audit records are preserved.
-- Relevant pending applicants are notified when required.</x:v>
+        <x:v>- Only the ACTIVE creator may delete and explicit confirmation is required.
+- Deletion is terminal, sets ProjectStatus = DELETED and deletedAt in UTC, and ordinary endpoints return 404.
+- Project, skills, applications, memberships, and audit records are preserved.
+- Every PENDING application becomes CANCELLED_PROJECT_DELETED atomically.
+- Each affected applicant receives exactly one PROJECT_DELETED notification.
+- The Project-owned anonymization hook redacts creator attribution and applies the same deletion/cancellation behavior.</x:v>
       </x:c>
       <x:c r="K47" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L47" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M47" s="16"/>
       <x:c r="N47" s="16"/>
@@ -63501,9 +63499,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f53d800d3e64eeb"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a0ac3141c654ea9"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dee722995414b4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85d841ae4ad3423a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66257,7 +66255,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0eae1a1dbbc4ba0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re11bc2c09cf54578"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66543,7 +66541,7 @@
         <x:v>Projects</x:v>
       </x:c>
       <x:c r="C25" s="31" t="str">
-        <x:v>teamSizeLimit includes the creator and is at least 2; open positions are derived from memberships.</x:v>
+        <x:v>Only ACTIVE, non-anonymized STUDENT accounts use Project recruitment. teamSizeLimit includes the creator and is at least 2; membership count, vacancies, fullness, expiry, and availability are derived, never stored as FULL.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -66554,7 +66552,7 @@
         <x:v>Projects</x:v>
       </x:c>
       <x:c r="C26" s="31" t="str">
-        <x:v>Project creation adds the CREATOR membership atomically; acceptance adds a TEAMMATE membership atomically while capacity remains.</x:v>
+        <x:v>Project creation atomically adds the sole CREATOR membership. One lifetime application exists per student/project. Acceptance atomically rechecks eligibility and capacity, creates one TEAMMATE membership, audits, and notifies without duplicate effects on identical retries.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -66565,7 +66563,7 @@
         <x:v>Projects</x:v>
       </x:c>
       <x:c r="C27" s="31" t="str">
-        <x:v>Closing blocks new applications but permits review of pre-closing pending applications while capacity remains.</x:v>
+        <x:v>applicationDeadline is mandatory and valid through that day in Asia/Dhaka. Default browse excludes expired OPEN projects but includes full OPEN projects; stored status and derived availability are independent AND-combined filters. Closed and expired projects retain direct details.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -66576,7 +66574,7 @@
         <x:v>Projects</x:v>
       </x:c>
       <x:c r="C28" s="31" t="str">
-        <x:v>Project deletion is soft and preserves applications, memberships, and audit history.</x:v>
+        <x:v>Creator-only soft deletion is terminal, preserves history, cancels pending applications, and notifies each affected applicant once. The Project-owned anonymization hook redacts attribution and performs the same deletion behavior; ordinary deleted-project endpoints return 404.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -66912,7 +66910,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc76e8da9183d48ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2af714576a642a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66977,7 +66975,7 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="D5" s="115" t="str">
-        <x:v>The baseline now contains explicit announcement draft, publication, unpublishing and expiry behavior; a separate Event lifecycle; terminal account anonymization; restoration of Club publishing; and the approved bounded content-reporting lifecycle. Warnings and unavailable project/career report targets remain deferred until their owning policies and modules are approved.</x:v>
+        <x:v>The baseline includes the implemented Project Teammate Finder core lifecycle, explicit derived availability and deadline rules, terminal project deletion, and the project-owned anonymization hook. Standalone candidate search, recommendation scoring, project reporting, member administration, warnings, and other deferred workflows remain outside the verified milestone.</x:v>
       </x:c>
       <x:c r="E5" s="116"/>
       <x:c r="F5" s="116"/>
@@ -67324,10 +67322,10 @@
         <x:v>FR_29–FR_39, FR_77</x:v>
       </x:c>
       <x:c r="D10" s="30" t="str">
-        <x:v>Create/browse/apply/review/close project recruitment</x:v>
+        <x:v>Core backend complete: create/browse/detail/edit/apply/review/close/reopen/delete, memberships, audits, notifications</x:v>
       </x:c>
       <x:c r="E10" s="30" t="str">
-        <x:v>Moved from MUST to SHOULD by team decision.</x:v>
+        <x:v>Standalone candidate search, recommendation scoring, project reporting, member leave/removal, ownership transfer, attachments, Flutter, and automatic chat creation remain deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -67466,7 +67464,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c17866468044af1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f4fa081c07a4a9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(project): add recruitment and team membership (#77) (#78)
</commit_message>
<xml_diff>
--- a/docs/requirements/UniConnect_Requirements_Baseline.xlsx
+++ b/docs/requirements/UniConnect_Requirements_Baseline.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="R69afee22b363497e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Rdd512aa099184a48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="R452a5338ad554aa2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="Re70a34437f6244e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="R51536b33cf5741b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="Rc2b91a1f0f8c4310"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="Rc05b016315274bf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Re2a21074ceed4a0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="R253303f188904593"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="R87d3e2b5a8454eba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="Rf4faa6cd2798456e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="Raa032e71943d4aac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -30450,7 +30450,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="L35" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>To Do</x:v>
       </x:c>
       <x:c r="M35" s="16"/>
       <x:c r="N35" s="16"/>
@@ -30509,7 +30509,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="L36" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>To Do</x:v>
       </x:c>
       <x:c r="M36" s="16"/>
       <x:c r="N36" s="16"/>
@@ -30570,7 +30570,7 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="L37" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>To Do</x:v>
       </x:c>
       <x:c r="M37" s="16"/>
       <x:c r="N37" s="16"/>
@@ -30591,7 +30591,7 @@
       <x:c r="AC37" s="16"/>
       <x:c r="AD37" s="16"/>
     </x:row>
-    <x:row r="38" ht="22.5" customHeight="1">
+    <x:row r="38" ht="156" hidden="0" customHeight="1">
       <x:c r="A38" s="11" t="n">
         <x:v>37</x:v>
       </x:c>
@@ -30620,17 +30620,18 @@
         <x:v>As a Student, I want to browse available project posts using filters and sorting options, so that I can find projects that match my skills and schedules efficiently.</x:v>
       </x:c>
       <x:c r="J38" s="13" t="str">
-        <x:v>- Open projects are displayed.
-- Skill, department, and status filters are available.
-- Sorting by date or deadline is available.
-- Project cards show key details.
-- Results are paginated.</x:v>
+        <x:v>- Default browse returns non-expired OPEN projects, including AVAILABLE and FULL projects.
+- Stored status and derived availability are separate filters and combine with AND.
+- Availability values are AVAILABLE, FULL, EXPIRED, and CLOSED.
+- Skill and creator-current-department filters are available.
+- Sorting supports newest-created and earliest-deadline order.
+- Results are paginated; DELETED projects never appear.</x:v>
       </x:c>
       <x:c r="K38" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L38" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M38" s="16"/>
       <x:c r="N38" s="16"/>
@@ -30651,7 +30652,7 @@
       <x:c r="AC38" s="16"/>
       <x:c r="AD38" s="16"/>
     </x:row>
-    <x:row r="39" ht="22.5" customHeight="1">
+    <x:row r="39" ht="132" hidden="0" customHeight="1">
       <x:c r="A39" s="11" t="n">
         <x:v>38</x:v>
       </x:c>
@@ -30680,17 +30681,17 @@
         <x:v>As a Student, I want to view the complete information of a selected project post, so that I can fully understand the project scope and requirements before deciding to join.</x:v>
       </x:c>
       <x:c r="J39" s="13" t="str">
-        <x:v>- Title and description are shown.
-- Required skills are shown.
-- Creator is shown.
-- Remaining positions are shown.
-- Current application status is shown.</x:v>
+        <x:v>- Title, description, skills, creator attribution, deadline, and lifecycle status are shown.
+- Membership count, vacancies, fullness, and availability are derived.
+- The current Student's lifetime application status is shown when one exists.
+- Closed and expired projects retain direct details.
+- DELETED projects return 404 from ordinary endpoints.</x:v>
       </x:c>
       <x:c r="K39" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L39" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M39" s="16"/>
       <x:c r="N39" s="16"/>
@@ -30711,7 +30712,7 @@
       <x:c r="AC39" s="16"/>
       <x:c r="AD39" s="16"/>
     </x:row>
-    <x:row r="40" ht="22.5" customHeight="1">
+    <x:row r="40" ht="156" hidden="0" customHeight="1">
       <x:c r="A40" s="11" t="n">
         <x:v>39</x:v>
       </x:c>
@@ -30740,18 +30741,18 @@
         <x:v>As a Student, I want to create a project post containing project details and required skills, so that I can attract suitable teammates who can contribute to my project.</x:v>
       </x:c>
       <x:c r="J40" s="13" t="str">
-        <x:v>- Title and description are required.
-- At least one required skill is selected.
-- teamSizeLimit is total capacity including the creator and is at least 2.
-- The Project is created with ProjectStatus = OPEN.
-- Creation atomically creates the sole CREATOR ProjectMembership.
-- openPositionCount is calculated from teamSizeLimit minus current memberships.</x:v>
+        <x:v>- Only an ACTIVE, non-anonymized STUDENT may create.
+- Title, description, applicationDeadline, and at least one required skill are required.
+- teamSizeLimit is total capacity including the creator and is between 2 and 100.
+- The deadline is valid through that date in Asia/Dhaka.
+- ProjectStatus is OPEN and the sole CREATOR membership is created atomically.
+- Membership count, vacancies, fullness, expiry, and availability are derived rather than stored.</x:v>
       </x:c>
       <x:c r="K40" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L40" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M40" s="16"/>
       <x:c r="N40" s="16"/>
@@ -30772,7 +30773,7 @@
       <x:c r="AC40" s="16"/>
       <x:c r="AD40" s="16"/>
     </x:row>
-    <x:row r="41" ht="22.5" customHeight="1">
+    <x:row r="41" ht="180" hidden="0" customHeight="1">
       <x:c r="A41" s="11" t="n">
         <x:v>40</x:v>
       </x:c>
@@ -30801,18 +30802,18 @@
         <x:v>As an eligible Student, I want to apply to an open project, so that I can join projects that interest me and fit my skills.</x:v>
       </x:c>
       <x:c r="J41" s="13" t="str">
-        <x:v>- The applicant has PlatformRole = STUDENT and AccountStatus = ACTIVE.
-- The Project is OPEN and has not been soft-deleted.
-- The creator and existing members cannot apply.
-- At most one application exists for the project/applicant pair.
-- The optional message is limited to 500 characters.
-- A valid application is stored as PENDING.</x:v>
+        <x:v>- Applicant and creator are currently ACTIVE, non-anonymized STUDENT accounts.
+- Project is OPEN, non-expired, not DELETED, and has a vacancy.
+- Creator and existing members cannot apply.
+- Exactly one lifetime application exists per project/applicant pair; withdrawal and reapplication are unavailable.
+- Optional message is at most 500 characters.
+- A valid application is stored as PENDING; the creator receives no application-received notification.</x:v>
       </x:c>
       <x:c r="K41" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L41" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M41" s="16"/>
       <x:c r="N41" s="16"/>
@@ -30833,7 +30834,7 @@
       <x:c r="AC41" s="16"/>
       <x:c r="AD41" s="16"/>
     </x:row>
-    <x:row r="42" ht="22.5" customHeight="1">
+    <x:row r="42" ht="96" hidden="0" customHeight="1">
       <x:c r="A42" s="11" t="n">
         <x:v>41</x:v>
       </x:c>
@@ -30862,17 +30863,16 @@
         <x:v>As the creator of a project, I want to view applications submitted to that project, so that I can review interested students and evaluate their suitability.</x:v>
       </x:c>
       <x:c r="J42" s="13" t="str">
-        <x:v>- Only the creator can view applications.
-- Application status is visible.
-- Applicant profile summary is shown.
-- Applicant message is shown.
-- Applications can be ordered by time.</x:v>
+        <x:v>- Only the ACTIVE creator may view applications.
+- Pending applications remain visible and reviewable after closing or expiry.
+- Applicant attribution, message, status, and UTC lifecycle timestamps are shown.
+- Deleted projects return 404 from ordinary endpoints.</x:v>
       </x:c>
       <x:c r="K42" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L42" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M42" s="16"/>
       <x:c r="N42" s="16"/>
@@ -30893,7 +30893,7 @@
       <x:c r="AC42" s="16"/>
       <x:c r="AD42" s="16"/>
     </x:row>
-    <x:row r="43" ht="22.5" customHeight="1">
+    <x:row r="43" ht="180" hidden="0" customHeight="1">
       <x:c r="A43" s="11" t="n">
         <x:v>42</x:v>
       </x:c>
@@ -30922,18 +30922,18 @@
         <x:v>As the creator of a project, I want to accept suitable applicants and decline unsuitable ones, so that I can select the best candidates for my team.</x:v>
       </x:c>
       <x:c r="J43" s="13" t="str">
-        <x:v>- Only the Project's creator may process an application.
-- Only PENDING applications may transition to ACCEPTED or REJECTED.
-- Acceptance atomically rechecks capacity, changes the application to ACCEPTED, and creates one TEAMMATE ProjectMembership.
-- Acceptance fails without partial change when capacity is full.
-- Rejection changes the application to REJECTED without creating membership.
-- The applicant receives one decision notification.</x:v>
+        <x:v>- Only the ACTIVE creator may process an application.
+- Only PENDING transitions to ACCEPTED or REJECTED; identical retries return the existing result.
+- Acceptance atomically locks, rechecks applicant eligibility and capacity, creates one TEAMMATE membership, audits, and notifies.
+- Capacity cannot be exceeded and partial acceptance cannot commit.
+- Rejection audits and notifies without membership.
+- Conflicting terminal retries return 409; identical retries duplicate nothing.</x:v>
       </x:c>
       <x:c r="K43" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L43" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M43" s="16"/>
       <x:c r="N43" s="16"/>
@@ -30954,7 +30954,7 @@
       <x:c r="AC43" s="16"/>
       <x:c r="AD43" s="16"/>
     </x:row>
-    <x:row r="44" ht="22.5" customHeight="1">
+    <x:row r="44" ht="108" hidden="0" customHeight="1">
       <x:c r="A44" s="11" t="n">
         <x:v>43</x:v>
       </x:c>
@@ -30983,17 +30983,17 @@
         <x:v>As the creator of a project, I want to update the project post, so that I can keep project details accurate and relevant for the future applicants.</x:v>
       </x:c>
       <x:c r="J44" s="13" t="str">
-        <x:v>- Only creator can edit.
-- Current values are shown.
-- Required fields cannot be removed.
-- Invalid values are rejected.
-- Valid changes appear immediately.</x:v>
+        <x:v>- Only the ACTIVE creator may edit a non-deleted OPEN or CLOSED Project.
+- Required fields remain valid and at least one skill remains required.
+- teamSizeLimit cannot be reduced below current membership.
+- Lifecycle timestamps are UTC.
+- Extending an OPEN Project's deadline can restore application availability.</x:v>
       </x:c>
       <x:c r="K44" s="15" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="L44" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M44" s="16"/>
       <x:c r="N44" s="16"/>
@@ -31014,7 +31014,7 @@
       <x:c r="AC44" s="16"/>
       <x:c r="AD44" s="16"/>
     </x:row>
-    <x:row r="45" ht="22.5" customHeight="1">
+    <x:row r="45" ht="132" hidden="0" customHeight="1">
       <x:c r="A45" s="11" t="n">
         <x:v>44</x:v>
       </x:c>
@@ -31043,18 +31043,17 @@
         <x:v>As a Project Creator whose available positions are filled, I want to close recruitment so that students do not spend time applying to an unavailable project.</x:v>
       </x:c>
       <x:c r="J45" s="13" t="str">
-        <x:v>- Only the creator may close an OPEN Project.
-- Closing changes ProjectStatus to CLOSED and rejects new applications.
-- Applications submitted before closing remain reviewable.
-- A pending pre-closing application may be accepted only while capacity remains.
-- The Project remains visible unless separately soft-deleted.
-- Closed recruitment is clearly displayed.</x:v>
+        <x:v>- Only the ACTIVE creator may close a non-deleted Project.
+- Closing is idempotent, sets ProjectStatus = CLOSED, records closedAt in UTC, and blocks new applications.
+- Pending pre-closing applications remain reviewable after close or expiry.
+- Acceptance remains possible only while capacity and applicant eligibility permit.
+- Closed projects retain direct details and explicit status/availability-filter browsing.</x:v>
       </x:c>
       <x:c r="K45" s="15" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="L45" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M45" s="16"/>
       <x:c r="N45" s="16"/>
@@ -31075,7 +31074,7 @@
       <x:c r="AC45" s="16"/>
       <x:c r="AD45" s="16"/>
     </x:row>
-    <x:row r="46" ht="22.5" customHeight="1">
+    <x:row r="46" ht="108" hidden="0" customHeight="1">
       <x:c r="A46" s="11" t="n">
         <x:v>45</x:v>
       </x:c>
@@ -31104,17 +31103,16 @@
         <x:v>As a Project Creator whose team has gained another vacancy, I want to reopen recruitment so that new candidates can apply.</x:v>
       </x:c>
       <x:c r="J46" s="13" t="str">
-        <x:v>- Only the creator may reopen the Project.
-- The Project is CLOSED, not DELETED, and has at least one derived open position.
-- Reopening changes ProjectStatus to OPEN.
-- New applications are accepted after reopening.
-- The Project returns to open-project browse results.</x:v>
+        <x:v>- Only the ACTIVE creator may reopen.
+- Project is CLOSED, non-deleted, has at least one vacancy, and has a deadline valid today or later in Asia/Dhaka.
+- Reopening changes ProjectStatus to OPEN and clears closedAt.
+- New applications become available only while the project remains non-expired and not full.</x:v>
       </x:c>
       <x:c r="K46" s="15" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="L46" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M46" s="16"/>
       <x:c r="N46" s="16"/>
@@ -31135,7 +31133,7 @@
       <x:c r="AC46" s="16"/>
       <x:c r="AD46" s="16"/>
     </x:row>
-    <x:row r="47" ht="22.5" customHeight="1">
+    <x:row r="47" ht="168" hidden="0" customHeight="1">
       <x:c r="A47" s="11" t="n">
         <x:v>46</x:v>
       </x:c>
@@ -31164,18 +31162,18 @@
         <x:v>As the creator of a Project, I want to remove it from normal use after confirmation so that outdated or abandoned projects no longer appear while historical records are preserved.</x:v>
       </x:c>
       <x:c r="J47" s="13" t="str">
-        <x:v>- Only the creator may initiate deletion.
-- Explicit confirmation is required; cancelling leaves the Project unchanged.
-- Confirmation sets ProjectStatus = DELETED and deletedAt.
-- The Project disappears from normal browse and search.
-- Project, application, membership, and audit records are preserved.
-- Relevant pending applicants are notified when required.</x:v>
+        <x:v>- Only the ACTIVE creator may delete and explicit confirmation is required.
+- Deletion is terminal, sets ProjectStatus = DELETED and deletedAt in UTC, and ordinary endpoints return 404.
+- Project, skills, applications, memberships, and audit records are preserved.
+- Every PENDING application becomes CANCELLED_PROJECT_DELETED atomically.
+- Each affected applicant receives exactly one PROJECT_DELETED notification.
+- The Project-owned anonymization hook redacts creator attribution and applies the same deletion/cancellation behavior.</x:v>
       </x:c>
       <x:c r="K47" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L47" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M47" s="16"/>
       <x:c r="N47" s="16"/>
@@ -63501,9 +63499,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f53d800d3e64eeb"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a0ac3141c654ea9"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dee722995414b4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85d841ae4ad3423a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66257,7 +66255,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0eae1a1dbbc4ba0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re11bc2c09cf54578"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66543,7 +66541,7 @@
         <x:v>Projects</x:v>
       </x:c>
       <x:c r="C25" s="31" t="str">
-        <x:v>teamSizeLimit includes the creator and is at least 2; open positions are derived from memberships.</x:v>
+        <x:v>Only ACTIVE, non-anonymized STUDENT accounts use Project recruitment. teamSizeLimit includes the creator and is at least 2; membership count, vacancies, fullness, expiry, and availability are derived, never stored as FULL.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -66554,7 +66552,7 @@
         <x:v>Projects</x:v>
       </x:c>
       <x:c r="C26" s="31" t="str">
-        <x:v>Project creation adds the CREATOR membership atomically; acceptance adds a TEAMMATE membership atomically while capacity remains.</x:v>
+        <x:v>Project creation atomically adds the sole CREATOR membership. One lifetime application exists per student/project. Acceptance atomically rechecks eligibility and capacity, creates one TEAMMATE membership, audits, and notifies without duplicate effects on identical retries.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -66565,7 +66563,7 @@
         <x:v>Projects</x:v>
       </x:c>
       <x:c r="C27" s="31" t="str">
-        <x:v>Closing blocks new applications but permits review of pre-closing pending applications while capacity remains.</x:v>
+        <x:v>applicationDeadline is mandatory and valid through that day in Asia/Dhaka. Default browse excludes expired OPEN projects but includes full OPEN projects; stored status and derived availability are independent AND-combined filters. Closed and expired projects retain direct details.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -66576,7 +66574,7 @@
         <x:v>Projects</x:v>
       </x:c>
       <x:c r="C28" s="31" t="str">
-        <x:v>Project deletion is soft and preserves applications, memberships, and audit history.</x:v>
+        <x:v>Creator-only soft deletion is terminal, preserves history, cancels pending applications, and notifies each affected applicant once. The Project-owned anonymization hook redacts attribution and performs the same deletion behavior; ordinary deleted-project endpoints return 404.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -66912,7 +66910,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc76e8da9183d48ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2af714576a642a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66977,7 +66975,7 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="D5" s="115" t="str">
-        <x:v>The baseline now contains explicit announcement draft, publication, unpublishing and expiry behavior; a separate Event lifecycle; terminal account anonymization; restoration of Club publishing; and the approved bounded content-reporting lifecycle. Warnings and unavailable project/career report targets remain deferred until their owning policies and modules are approved.</x:v>
+        <x:v>The baseline includes the implemented Project Teammate Finder core lifecycle, explicit derived availability and deadline rules, terminal project deletion, and the project-owned anonymization hook. Standalone candidate search, recommendation scoring, project reporting, member administration, warnings, and other deferred workflows remain outside the verified milestone.</x:v>
       </x:c>
       <x:c r="E5" s="116"/>
       <x:c r="F5" s="116"/>
@@ -67324,10 +67322,10 @@
         <x:v>FR_29–FR_39, FR_77</x:v>
       </x:c>
       <x:c r="D10" s="30" t="str">
-        <x:v>Create/browse/apply/review/close project recruitment</x:v>
+        <x:v>Core backend complete: create/browse/detail/edit/apply/review/close/reopen/delete, memberships, audits, notifications</x:v>
       </x:c>
       <x:c r="E10" s="30" t="str">
-        <x:v>Moved from MUST to SHOULD by team decision.</x:v>
+        <x:v>Standalone candidate search, recommendation scoring, project reporting, member leave/removal, ownership transfer, attachments, Flutter, and automatic chat creation remain deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -67466,7 +67464,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c17866468044af1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f4fa081c07a4a9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(project): add privacy-aware candidate search (#83)
</commit_message>
<xml_diff>
--- a/docs/requirements/UniConnect_Requirements_Baseline.xlsx
+++ b/docs/requirements/UniConnect_Requirements_Baseline.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="Rc05b016315274bf9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Re2a21074ceed4a0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="R253303f188904593"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="R87d3e2b5a8454eba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="Rf4faa6cd2798456e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="Raa032e71943d4aac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="Rb41f6d50ed254479"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="R91cb37e2a07d44c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="Rabf5d226aa5f43cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="R30e9a608601c4308"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="R1687628f3e59444c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="R22f4adb1770d405b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -30439,18 +30439,19 @@
         <x:v>As a Student, I want to search for teammates with required skills, so that I can easily find people who have the expertise I need for my projects.</x:v>
       </x:c>
       <x:c r="J35" s="13" t="str">
-        <x:v>- At least one required skill is entered.
-- Search returns Students whose profiles contain the required skills.
-- Department, study year, and availability filters are available.
-- Results show the candidate's relevant skills.
-- Candidates who do not meet required-skill conditions are excluded or ranked lower according to the matching rule.
+        <x:v>- At least one required skill is entered; combined required and optional skills are limited to 10.
+- Candidates are ACTIVE, non-anonymized Students with permitted profiles containing every required skill.
+- Optional skills do not affect eligibility, counts, ordering, or pagination.
+- Department, study year, and project-availability filters are available and combine with AND.
+- Privacy applies before filtering, counting, ordering, and pagination.
+- Results show only the requested, visible skill intersection labelled REQUIRED or OPTIONAL.
 - Selecting a result opens the candidate's permitted profile.</x:v>
       </x:c>
       <x:c r="K35" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L35" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M35" s="16"/>
       <x:c r="N35" s="16"/>
@@ -30500,16 +30501,18 @@
         <x:v>As a Student who has not finalized a project idea, I want to discover people with complementary skills so that we can discuss possible projects before building a new project.</x:v>
       </x:c>
       <x:c r="J36" s="13" t="str">
-        <x:v>- The search can be performed without selecting or creating a project.
-- Multiple required or optional skills can be used for exploratory discovery.
-- Results can include candidates outside the searcher's existing connections.
-- The search does not create a project or application record.</x:v>
+        <x:v>- Search can be performed without selecting or creating a project.
+- Multiple required and optional skills can be used; at least one required skill remains mandatory.
+- Results can include candidates outside existing connections only when profile privacy permits their protected details.
+- Project-owned search uses stored project skills and excludes current members and all lifetime applicants.
+- Search creates no project, application, audit, notification, recommendation, or skill-vocabulary record.
+- Candidate matching and project availability do not restrict a Student's separate permission to apply.</x:v>
       </x:c>
       <x:c r="K36" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L36" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M36" s="16"/>
       <x:c r="N36" s="16"/>
@@ -63499,9 +63502,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a0ac3141c654ea9"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79b4351847c24dbf"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85d841ae4ad3423a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf2478bd2d994ab2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66255,7 +66258,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re11bc2c09cf54578"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R570049ebf7114f40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66910,7 +66913,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2af714576a642a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2af02ad9cd444f6c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66975,7 +66978,7 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="D5" s="115" t="str">
-        <x:v>The baseline includes the implemented Project Teammate Finder core lifecycle, explicit derived availability and deadline rules, terminal project deletion, and the project-owned anonymization hook. Standalone candidate search, recommendation scoring, project reporting, member administration, warnings, and other deferred workflows remain outside the verified milestone.</x:v>
+        <x:v>The baseline includes the implemented Project Teammate Finder core lifecycle and FR_29 candidate search with privacy-safe all-required-skill matching. FR_30 recommendation scoring, project reporting, member administration, warnings, and other deferred workflows remain outside the verified milestone.</x:v>
       </x:c>
       <x:c r="E5" s="116"/>
       <x:c r="F5" s="116"/>
@@ -67322,10 +67325,10 @@
         <x:v>FR_29–FR_39, FR_77</x:v>
       </x:c>
       <x:c r="D10" s="30" t="str">
-        <x:v>Core backend complete: create/browse/detail/edit/apply/review/close/reopen/delete, memberships, audits, notifications</x:v>
+        <x:v>Backend complete: candidate search, create/browse/detail/edit/apply/review/close/reopen/delete, memberships, audits, notifications</x:v>
       </x:c>
       <x:c r="E10" s="30" t="str">
-        <x:v>Standalone candidate search, recommendation scoring, project reporting, member leave/removal, ownership transfer, attachments, Flutter, and automatic chat creation remain deferred.</x:v>
+        <x:v>FR_30 recommendation scoring, project reporting, member leave/removal, ownership transfer, attachments, Flutter, and automatic chat creation remain deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -67464,7 +67467,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f4fa081c07a4a9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19cd099de9094bab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(project): add privacy-aware candidate search (#83) (#84)
</commit_message>
<xml_diff>
--- a/docs/requirements/UniConnect_Requirements_Baseline.xlsx
+++ b/docs/requirements/UniConnect_Requirements_Baseline.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="Rc05b016315274bf9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Re2a21074ceed4a0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="R253303f188904593"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="R87d3e2b5a8454eba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="Rf4faa6cd2798456e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="Raa032e71943d4aac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="Rb41f6d50ed254479"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="R91cb37e2a07d44c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="Rabf5d226aa5f43cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="R30e9a608601c4308"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="R1687628f3e59444c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="R22f4adb1770d405b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -30439,18 +30439,19 @@
         <x:v>As a Student, I want to search for teammates with required skills, so that I can easily find people who have the expertise I need for my projects.</x:v>
       </x:c>
       <x:c r="J35" s="13" t="str">
-        <x:v>- At least one required skill is entered.
-- Search returns Students whose profiles contain the required skills.
-- Department, study year, and availability filters are available.
-- Results show the candidate's relevant skills.
-- Candidates who do not meet required-skill conditions are excluded or ranked lower according to the matching rule.
+        <x:v>- At least one required skill is entered; combined required and optional skills are limited to 10.
+- Candidates are ACTIVE, non-anonymized Students with permitted profiles containing every required skill.
+- Optional skills do not affect eligibility, counts, ordering, or pagination.
+- Department, study year, and project-availability filters are available and combine with AND.
+- Privacy applies before filtering, counting, ordering, and pagination.
+- Results show only the requested, visible skill intersection labelled REQUIRED or OPTIONAL.
 - Selecting a result opens the candidate's permitted profile.</x:v>
       </x:c>
       <x:c r="K35" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L35" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M35" s="16"/>
       <x:c r="N35" s="16"/>
@@ -30500,16 +30501,18 @@
         <x:v>As a Student who has not finalized a project idea, I want to discover people with complementary skills so that we can discuss possible projects before building a new project.</x:v>
       </x:c>
       <x:c r="J36" s="13" t="str">
-        <x:v>- The search can be performed without selecting or creating a project.
-- Multiple required or optional skills can be used for exploratory discovery.
-- Results can include candidates outside the searcher's existing connections.
-- The search does not create a project or application record.</x:v>
+        <x:v>- Search can be performed without selecting or creating a project.
+- Multiple required and optional skills can be used; at least one required skill remains mandatory.
+- Results can include candidates outside existing connections only when profile privacy permits their protected details.
+- Project-owned search uses stored project skills and excludes current members and all lifetime applicants.
+- Search creates no project, application, audit, notification, recommendation, or skill-vocabulary record.
+- Candidate matching and project availability do not restrict a Student's separate permission to apply.</x:v>
       </x:c>
       <x:c r="K36" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L36" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M36" s="16"/>
       <x:c r="N36" s="16"/>
@@ -63499,9 +63502,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a0ac3141c654ea9"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79b4351847c24dbf"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85d841ae4ad3423a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf2478bd2d994ab2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66255,7 +66258,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re11bc2c09cf54578"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R570049ebf7114f40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66910,7 +66913,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2af714576a642a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2af02ad9cd444f6c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66975,7 +66978,7 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="D5" s="115" t="str">
-        <x:v>The baseline includes the implemented Project Teammate Finder core lifecycle, explicit derived availability and deadline rules, terminal project deletion, and the project-owned anonymization hook. Standalone candidate search, recommendation scoring, project reporting, member administration, warnings, and other deferred workflows remain outside the verified milestone.</x:v>
+        <x:v>The baseline includes the implemented Project Teammate Finder core lifecycle and FR_29 candidate search with privacy-safe all-required-skill matching. FR_30 recommendation scoring, project reporting, member administration, warnings, and other deferred workflows remain outside the verified milestone.</x:v>
       </x:c>
       <x:c r="E5" s="116"/>
       <x:c r="F5" s="116"/>
@@ -67322,10 +67325,10 @@
         <x:v>FR_29–FR_39, FR_77</x:v>
       </x:c>
       <x:c r="D10" s="30" t="str">
-        <x:v>Core backend complete: create/browse/detail/edit/apply/review/close/reopen/delete, memberships, audits, notifications</x:v>
+        <x:v>Backend complete: candidate search, create/browse/detail/edit/apply/review/close/reopen/delete, memberships, audits, notifications</x:v>
       </x:c>
       <x:c r="E10" s="30" t="str">
-        <x:v>Standalone candidate search, recommendation scoring, project reporting, member leave/removal, ownership transfer, attachments, Flutter, and automatic chat creation remain deferred.</x:v>
+        <x:v>FR_30 recommendation scoring, project reporting, member leave/removal, ownership transfer, attachments, Flutter, and automatic chat creation remain deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -67464,7 +67467,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f4fa081c07a4a9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19cd099de9094bab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(project): add explainable recommendation scoring (#85)
</commit_message>
<xml_diff>
--- a/docs/requirements/UniConnect_Requirements_Baseline.xlsx
+++ b/docs/requirements/UniConnect_Requirements_Baseline.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="Rb41f6d50ed254479"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="R91cb37e2a07d44c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="Rabf5d226aa5f43cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="R30e9a608601c4308"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="R1687628f3e59444c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="R22f4adb1770d405b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="Rc0aa79f1207741f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Rc87224aa9cc84c38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="Re8b3c1ae094d4e25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="R9208092dcec44d27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="Rad849eb0f0ea49d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="Rffa5a778a7cb40a5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -30553,7 +30553,7 @@
         <x:v>Student</x:v>
       </x:c>
       <x:c r="G37" s="19" t="str">
-        <x:v>to receive recommendations for potential teammates based on skill compatibility, connection proximity, and intereststo receive recommendations for potential teammates based on skills, connection proximity, and interests</x:v>
+        <x:v>to receive recommendations for potential teammates based on skills, direct connection, and interests</x:v>
       </x:c>
       <x:c r="H37" s="19" t="str">
         <x:v>I can discover well-matched collaborators.</x:v>
@@ -30562,18 +30562,18 @@
         <x:v>As a Student, I want to receive recommendations for potential teammates based on skills, connection proximity, and interests, so that I can discover well-matched collaborators.</x:v>
       </x:c>
       <x:c r="J37" s="13" t="str">
-        <x:v>- Eligible candidates are ACTIVE STUDENT users who are project-available and otherwise permitted.
-- Each candidate receives a calculated 0–100% score.
-- Required skills, connection proximity, and interests contribute to the score.
-- Results are ordered highest to lowest.
-- Fixed scoring weights are not stored unless separately approved as a business rule.
-- Recommendation results are not permanent domain entities.</x:v>
+        <x:v>- Only the ACTIVE, non-anonymized STUDENT project creator may request recommendations. Missing, deleted, or non-owned projects return the canonical 404; closed, expired, or full projects return an empty array.
+- Eligible candidates are ACTIVE, non-anonymized STUDENT users with a student profile, projectAvailable=true, and profile details visible to the creator. Exclude the creator, current members, and every lifetime applicant.
+- A candidate must match at least one required project skill; partial required-skill matches remain eligible. Projects with no required skills return an empty array.
+- Score = skillPoints + interestPoints + connectionPoints, calculated transiently from visible data and never persisted. Skills contribute up to 70 points using weight 3 per required skill and weight 1 per optional skill. Interests contribute up to 20 points as visible normalized intersection divided by the creator's normalized interest count. An ACCEPTED direct connection contributes 10 points. Missing components are not redistributed.
+- Rank all eligible candidates by the unrounded total descending, then normalized case-insensitive name and user ID; return at most 20. Display scores and components to two decimals using HALF_UP. Independently rounded components may differ from the rounded total by 0.01.
+- The array response retains matched required and optional skills and adds score, component points, matched interests, and directlyConnected. Explanations expose only data visible to the creator. Recommendation matching does not restrict application eligibility.</x:v>
       </x:c>
       <x:c r="K37" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L37" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M37" s="16"/>
       <x:c r="N37" s="16"/>
@@ -63502,9 +63502,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79b4351847c24dbf"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd2636db2bf6489e"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf2478bd2d994ab2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re673403394de4489"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -64588,7 +64588,7 @@
         <x:v>Reworded</x:v>
       </x:c>
       <x:c r="G37" s="31" t="str">
-        <x:v>Presented recommendations as stored behavior with implied but unconfirmed fixed weighting.</x:v>
+        <x:v>Approved transient scoring now uses explicit 70-point weighted skills, 20-point visible interest overlap, and 10-point accepted direct-connection components.</x:v>
       </x:c>
       <x:c r="H37" s="31" t="str">
         <x:v>Made recommendations calculated/transient while retaining the confirmed factors.</x:v>
@@ -66258,7 +66258,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R570049ebf7114f40"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7597c85729464539"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66913,7 +66913,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2af02ad9cd444f6c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d991c7719384a72"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66978,7 +66978,7 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="D5" s="115" t="str">
-        <x:v>The baseline includes the implemented Project Teammate Finder core lifecycle and FR_29 candidate search with privacy-safe all-required-skill matching. FR_30 recommendation scoring, project reporting, member administration, warnings, and other deferred workflows remain outside the verified milestone.</x:v>
+        <x:v>The baseline includes the implemented Project Teammate Finder core lifecycle, FR_29 privacy-safe all-required-skill candidate search, and FR_30 transient weighted recommendations. Project reporting, member administration, warnings, and other deferred workflows remain outside the verified milestone.</x:v>
       </x:c>
       <x:c r="E5" s="116"/>
       <x:c r="F5" s="116"/>
@@ -67325,10 +67325,10 @@
         <x:v>FR_29–FR_39, FR_77</x:v>
       </x:c>
       <x:c r="D10" s="30" t="str">
-        <x:v>Backend complete: candidate search, create/browse/detail/edit/apply/review/close/reopen/delete, memberships, audits, notifications</x:v>
+        <x:v>Backend complete: candidate search, transient recommendations, create/browse/detail/edit/apply/review/close/reopen/delete, memberships, audits, notifications</x:v>
       </x:c>
       <x:c r="E10" s="30" t="str">
-        <x:v>FR_30 recommendation scoring, project reporting, member leave/removal, ownership transfer, attachments, Flutter, and automatic chat creation remain deferred.</x:v>
+        <x:v>Project reporting, member leave/removal, ownership transfer, attachments, Flutter score display, and automatic chat creation remain deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -67467,7 +67467,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19cd099de9094bab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a1c775bd13c4585"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(project): add explainable recommendation scoring (#85) (#86)
</commit_message>
<xml_diff>
--- a/docs/requirements/UniConnect_Requirements_Baseline.xlsx
+++ b/docs/requirements/UniConnect_Requirements_Baseline.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="Rb41f6d50ed254479"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="R91cb37e2a07d44c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="Rabf5d226aa5f43cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="R30e9a608601c4308"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="R1687628f3e59444c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="R22f4adb1770d405b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="Rc0aa79f1207741f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Rc87224aa9cc84c38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="Re8b3c1ae094d4e25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="R9208092dcec44d27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="Rad849eb0f0ea49d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="Rffa5a778a7cb40a5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -30553,7 +30553,7 @@
         <x:v>Student</x:v>
       </x:c>
       <x:c r="G37" s="19" t="str">
-        <x:v>to receive recommendations for potential teammates based on skill compatibility, connection proximity, and intereststo receive recommendations for potential teammates based on skills, connection proximity, and interests</x:v>
+        <x:v>to receive recommendations for potential teammates based on skills, direct connection, and interests</x:v>
       </x:c>
       <x:c r="H37" s="19" t="str">
         <x:v>I can discover well-matched collaborators.</x:v>
@@ -30562,18 +30562,18 @@
         <x:v>As a Student, I want to receive recommendations for potential teammates based on skills, connection proximity, and interests, so that I can discover well-matched collaborators.</x:v>
       </x:c>
       <x:c r="J37" s="13" t="str">
-        <x:v>- Eligible candidates are ACTIVE STUDENT users who are project-available and otherwise permitted.
-- Each candidate receives a calculated 0–100% score.
-- Required skills, connection proximity, and interests contribute to the score.
-- Results are ordered highest to lowest.
-- Fixed scoring weights are not stored unless separately approved as a business rule.
-- Recommendation results are not permanent domain entities.</x:v>
+        <x:v>- Only the ACTIVE, non-anonymized STUDENT project creator may request recommendations. Missing, deleted, or non-owned projects return the canonical 404; closed, expired, or full projects return an empty array.
+- Eligible candidates are ACTIVE, non-anonymized STUDENT users with a student profile, projectAvailable=true, and profile details visible to the creator. Exclude the creator, current members, and every lifetime applicant.
+- A candidate must match at least one required project skill; partial required-skill matches remain eligible. Projects with no required skills return an empty array.
+- Score = skillPoints + interestPoints + connectionPoints, calculated transiently from visible data and never persisted. Skills contribute up to 70 points using weight 3 per required skill and weight 1 per optional skill. Interests contribute up to 20 points as visible normalized intersection divided by the creator's normalized interest count. An ACCEPTED direct connection contributes 10 points. Missing components are not redistributed.
+- Rank all eligible candidates by the unrounded total descending, then normalized case-insensitive name and user ID; return at most 20. Display scores and components to two decimals using HALF_UP. Independently rounded components may differ from the rounded total by 0.01.
+- The array response retains matched required and optional skills and adds score, component points, matched interests, and directlyConnected. Explanations expose only data visible to the creator. Recommendation matching does not restrict application eligibility.</x:v>
       </x:c>
       <x:c r="K37" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L37" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M37" s="16"/>
       <x:c r="N37" s="16"/>
@@ -63502,9 +63502,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79b4351847c24dbf"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd2636db2bf6489e"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf2478bd2d994ab2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re673403394de4489"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -64588,7 +64588,7 @@
         <x:v>Reworded</x:v>
       </x:c>
       <x:c r="G37" s="31" t="str">
-        <x:v>Presented recommendations as stored behavior with implied but unconfirmed fixed weighting.</x:v>
+        <x:v>Approved transient scoring now uses explicit 70-point weighted skills, 20-point visible interest overlap, and 10-point accepted direct-connection components.</x:v>
       </x:c>
       <x:c r="H37" s="31" t="str">
         <x:v>Made recommendations calculated/transient while retaining the confirmed factors.</x:v>
@@ -66258,7 +66258,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R570049ebf7114f40"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7597c85729464539"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66913,7 +66913,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2af02ad9cd444f6c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d991c7719384a72"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66978,7 +66978,7 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="D5" s="115" t="str">
-        <x:v>The baseline includes the implemented Project Teammate Finder core lifecycle and FR_29 candidate search with privacy-safe all-required-skill matching. FR_30 recommendation scoring, project reporting, member administration, warnings, and other deferred workflows remain outside the verified milestone.</x:v>
+        <x:v>The baseline includes the implemented Project Teammate Finder core lifecycle, FR_29 privacy-safe all-required-skill candidate search, and FR_30 transient weighted recommendations. Project reporting, member administration, warnings, and other deferred workflows remain outside the verified milestone.</x:v>
       </x:c>
       <x:c r="E5" s="116"/>
       <x:c r="F5" s="116"/>
@@ -67325,10 +67325,10 @@
         <x:v>FR_29–FR_39, FR_77</x:v>
       </x:c>
       <x:c r="D10" s="30" t="str">
-        <x:v>Backend complete: candidate search, create/browse/detail/edit/apply/review/close/reopen/delete, memberships, audits, notifications</x:v>
+        <x:v>Backend complete: candidate search, transient recommendations, create/browse/detail/edit/apply/review/close/reopen/delete, memberships, audits, notifications</x:v>
       </x:c>
       <x:c r="E10" s="30" t="str">
-        <x:v>FR_30 recommendation scoring, project reporting, member leave/removal, ownership transfer, attachments, Flutter, and automatic chat creation remain deferred.</x:v>
+        <x:v>Project reporting, member leave/removal, ownership transfer, attachments, Flutter score display, and automatic chat creation remain deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -67467,7 +67467,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19cd099de9094bab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a1c775bd13c4585"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(reporting): support project and career-post reports (#87)
</commit_message>
<xml_diff>
--- a/docs/requirements/UniConnect_Requirements_Baseline.xlsx
+++ b/docs/requirements/UniConnect_Requirements_Baseline.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="Rc0aa79f1207741f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Rc87224aa9cc84c38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="Re8b3c1ae094d4e25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="R9208092dcec44d27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="Rad849eb0f0ea49d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="Rffa5a778a7cb40a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="R7396c94319d84e2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Rf732b2422803441e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="Ra1685a0350ec4973"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="Rbb3dad68a9a644c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="Re89c0b7117744b83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="Rc06ba44a6d824f1e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -32864,9 +32864,10 @@
       </x:c>
       <x:c r="J75" s="13" t="str">
         <x:v>- Any authenticated ACTIVE, non-anonymized user may submit regardless of selected context.
-- Supported targets are USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE; projects and career posts remain deferred until their modules exist.
-- The reporter must be able to access the target; inaccessible and nonexistent targets both return 404.
-- Minimal immutable evidence is captured through the owning module and is never returned in reporter DTOs.
+- Supported targets are USER, CLUB, ANNOUNCEMENT, EVENT, CHAT_MESSAGE, PROJECT, and CAREER_POST.
+- The reporter must be able to access the target through its owning module; inaccessible and nonexistent targets both return 404. Closed/expired Project or Career content remains reportable only while ordinary detail remains accessible.
+- Project reporting does not require Student, apply, membership, edit, or management eligibility; Career reporting does not require save, apply, edit, or management eligibility.
+- Minimal immutable evidence contains only ordinary reporter-visible fields, captures the Project creator or Career author as owner, and is never returned in reporter DTOs.
 - One open report is allowed per reporter and target; different reporters remain independent and a later report is allowed after closure.
 - Lifecycle is SUBMITTED → UNDER_REVIEW → ACTION_TAKEN or NO_ACTION.
 - The first SYSTEM_ADMINISTRATION reviewer owns resolution; concurrent claims and decisions cannot overwrite each other.
@@ -32878,7 +32879,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="L75" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M75" s="16"/>
       <x:c r="N75" s="16"/>
@@ -32933,15 +32934,17 @@
 - CLUB accepts publishing suspension or removal of that club.
 - ANNOUNCEMENT and EVENT accept removal by an existing authorized club operator, suspension of the captured author, or publishing suspension/removal of the captured parent club.
 - CHAT_MESSAGE accepts suspension of the captured sender.
-- Server-side checks verify the retained audit, target/author/club relationship, and that the action was not already reversed at resolution time.
-- Existing permissions for account, club, and publication actions remain unchanged; no administrative chat hiding, warning, or new publication-removal permission is created.
+- PROJECT accepts only an existing suspension of the captured creator.
+- CAREER_POST accepts only an existing suspension of the captured author.
+- Server-side checks verify the retained audit, target/owner relationship, temporal validity, and that the suspension was not reversed at resolution time; evidence linking serializes with reversal.
+- Existing permissions remain unchanged; no project/career removal, administrative chat hiding, warning, or new publication-removal permission is created.
 - Historical action identity remains linked if the action is reversed later.</x:v>
       </x:c>
       <x:c r="K76" s="15" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="L76" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M76" s="16"/>
       <x:c r="N76" s="16"/>
@@ -63502,9 +63505,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd2636db2bf6489e"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcf4afed417a4af2"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re673403394de4489"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c196f0c502d4659"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -65693,10 +65696,10 @@
         <x:v>Content reporting previously lacked approved target, access, lifecycle, concurrency, evidence, privacy, and notification rules.</x:v>
       </x:c>
       <x:c r="H75" s="31" t="str">
-        <x:v>Approved the bounded USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE reporting lifecycle with owner-only reporter reads and SYSTEM_ADMINISTRATION review.</x:v>
+        <x:v>Implemented the USER, CLUB, ANNOUNCEMENT, EVENT, CHAT_MESSAGE, PROJECT, and CAREER_POST reporting lifecycle with owner-only reporter reads and SYSTEM_ADMINISTRATION review.</x:v>
       </x:c>
       <x:c r="I75" s="31" t="str">
-        <x:v>Administration_Notification.drawio; One_to_One_Chat.drawio; CONTENT_REPORTING.md</x:v>
+        <x:v>Administration_Notification.drawio; One_to_One_Chat.drawio; Project_Teammate_Finder.drawio; Career_Board.drawio; CONTENT_REPORTING.md</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -65722,10 +65725,10 @@
         <x:v>The prior wording granted generic SYSTEM_ADMIN content-removal authority and referenced unavailable Project and JobPost modules.</x:v>
       </x:c>
       <x:c r="H76" s="31" t="str">
-        <x:v>Separated report resolution from action execution, retained existing action permissions, and required a verified link to qualifying committed evidence.</x:v>
+        <x:v>Separated report resolution from action execution, retained existing action permissions, and added verified owner-account suspension evidence for PROJECT and CAREER_POST without removal authority.</x:v>
       </x:c>
       <x:c r="I76" s="31" t="str">
-        <x:v>Administration_Notification.drawio; CONTENT_REPORTING.md</x:v>
+        <x:v>Administration_Notification.drawio; Project_Teammate_Finder.drawio; Career_Board.drawio; CONTENT_REPORTING.md</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -66258,7 +66261,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7597c85729464539"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R014003f93a0f4955"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66830,7 +66833,7 @@
         <x:v>Reporting</x:v>
       </x:c>
       <x:c r="C51" s="30" t="str">
-        <x:v>Supported targets are USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE. Project and career-post targets remain deferred until their modules exist.</x:v>
+        <x:v>Supported targets are USER, CLUB, ANNOUNCEMENT, EVENT, CHAT_MESSAGE, PROJECT, and CAREER_POST. Project and Career own ordinary detail access and safe immutable snapshots; accessible closed/expired content remains reportable, while missing, deleted, removed, or inaccessible targets return 404.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -66863,7 +66866,7 @@
         <x:v>Reporting</x:v>
       </x:c>
       <x:c r="C54" s="30" t="str">
-        <x:v>ACTION_TAKEN links an already committed qualifying action verified through the owning module; resolving a report never executes moderation.</x:v>
+        <x:v>ACTION_TAKEN links an already committed qualifying action verified through the owning module; resolving a report never executes moderation. PROJECT and CAREER_POST accept only an existing unreversed suspension of the captured creator/author.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -66907,13 +66910,13 @@
         <x:v>Reporting</x:v>
       </x:c>
       <x:c r="C58" s="30" t="str">
-        <x:v>Warnings, administrative chat hiding, and new publication-removal permissions are outside the bounded reporting phase.</x:v>
+        <x:v>Warnings, administrative chat hiding, new publication-removal permissions, and administrator project/career removal are outside the bounded reporting phase.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d991c7719384a72"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7672280eb674053"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66978,7 +66981,7 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="D5" s="115" t="str">
-        <x:v>The baseline includes the implemented Project Teammate Finder core lifecycle, FR_29 privacy-safe all-required-skill candidate search, and FR_30 transient weighted recommendations. Project reporting, member administration, warnings, and other deferred workflows remain outside the verified milestone.</x:v>
+        <x:v>The baseline includes the implemented Project Teammate Finder core lifecycle, FR_29 privacy-safe candidate search, FR_30 transient recommendations, Career Board, and backend content reporting for Project and Career posts. Member administration, warnings, Flutter reporting screens, and other deferred workflows remain outside the verified milestone.</x:v>
       </x:c>
       <x:c r="E5" s="116"/>
       <x:c r="F5" s="116"/>
@@ -67067,7 +67070,7 @@
         <x:v>FR_67–FR_68 — Content reporting</x:v>
       </x:c>
       <x:c r="B12" s="130" t="str">
-        <x:v>Approved bounded backend reporting for USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE with retained evidence, reviewer ownership, verified action links, reporter resolution notification, atomic history, and no action execution during resolution.</x:v>
+        <x:v>Implemented bounded backend reporting for USER, CLUB, ANNOUNCEMENT, EVENT, CHAT_MESSAGE, PROJECT, and CAREER_POST with retained evidence, reviewer ownership, verified action links, reporter resolution notification, atomic history, and no action execution during resolution. Project/Career ACTION_TAKEN evidence is limited to an unreversed suspension of the captured owner.</x:v>
       </x:c>
       <x:c r="C12" s="130"/>
       <x:c r="D12" s="130"/>
@@ -67328,7 +67331,7 @@
         <x:v>Backend complete: candidate search, transient recommendations, create/browse/detail/edit/apply/review/close/reopen/delete, memberships, audits, notifications</x:v>
       </x:c>
       <x:c r="E10" s="30" t="str">
-        <x:v>Project reporting, member leave/removal, ownership transfer, attachments, Flutter score display, and automatic chat creation remain deferred.</x:v>
+        <x:v>Project reporting is implemented. Member leave/removal, ownership transfer, attachments, Flutter score/report UI, and automatic chat creation remain deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -67342,10 +67345,10 @@
         <x:v>FR_56–FR_61, FR_81–FR_82</x:v>
       </x:c>
       <x:c r="D11" s="30" t="str">
-        <x:v>Publish, browse, save, edit and close career posts</x:v>
+        <x:v>Backend complete: publish, browse, detail, save, edit, close, retained closed/expired access, and content-report snapshot support</x:v>
       </x:c>
       <x:c r="E11" s="30" t="str">
-        <x:v>Implement after MUST modules are integrated.</x:v>
+        <x:v>Career-post reporting is implemented with captured-author suspension evidence only. Flutter screens, administrative removal, reopening, author deletion, and internal applications remain deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
@@ -67430,7 +67433,7 @@
         <x:v>Backend submission, retained evidence, administration review, verified action linking, audit, and resolution notification</x:v>
       </x:c>
       <x:c r="E16" s="30" t="str">
-        <x:v>Targets are USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE. Flutter screens and unavailable project/career targets remain separate.</x:v>
+        <x:v>Targets are USER, CLUB, ANNOUNCEMENT, EVENT, CHAT_MESSAGE, PROJECT, and CAREER_POST. Project/Career ACTION_TAKEN links only verified owner-account suspension. Flutter reporting screens remain separate.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" hidden="0" customHeight="1">
@@ -67467,7 +67470,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a1c775bd13c4585"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R841a103d19414817"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(reporting): support project and career-post reports (#87) (#88)
</commit_message>
<xml_diff>
--- a/docs/requirements/UniConnect_Requirements_Baseline.xlsx
+++ b/docs/requirements/UniConnect_Requirements_Baseline.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="Rc0aa79f1207741f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Rc87224aa9cc84c38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="Re8b3c1ae094d4e25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="R9208092dcec44d27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="Rad849eb0f0ea49d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="Rffa5a778a7cb40a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="R7396c94319d84e2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Rf732b2422803441e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="Ra1685a0350ec4973"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="Rbb3dad68a9a644c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="Re89c0b7117744b83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="Rc06ba44a6d824f1e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -32864,9 +32864,10 @@
       </x:c>
       <x:c r="J75" s="13" t="str">
         <x:v>- Any authenticated ACTIVE, non-anonymized user may submit regardless of selected context.
-- Supported targets are USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE; projects and career posts remain deferred until their modules exist.
-- The reporter must be able to access the target; inaccessible and nonexistent targets both return 404.
-- Minimal immutable evidence is captured through the owning module and is never returned in reporter DTOs.
+- Supported targets are USER, CLUB, ANNOUNCEMENT, EVENT, CHAT_MESSAGE, PROJECT, and CAREER_POST.
+- The reporter must be able to access the target through its owning module; inaccessible and nonexistent targets both return 404. Closed/expired Project or Career content remains reportable only while ordinary detail remains accessible.
+- Project reporting does not require Student, apply, membership, edit, or management eligibility; Career reporting does not require save, apply, edit, or management eligibility.
+- Minimal immutable evidence contains only ordinary reporter-visible fields, captures the Project creator or Career author as owner, and is never returned in reporter DTOs.
 - One open report is allowed per reporter and target; different reporters remain independent and a later report is allowed after closure.
 - Lifecycle is SUBMITTED → UNDER_REVIEW → ACTION_TAKEN or NO_ACTION.
 - The first SYSTEM_ADMINISTRATION reviewer owns resolution; concurrent claims and decisions cannot overwrite each other.
@@ -32878,7 +32879,7 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="L75" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M75" s="16"/>
       <x:c r="N75" s="16"/>
@@ -32933,15 +32934,17 @@
 - CLUB accepts publishing suspension or removal of that club.
 - ANNOUNCEMENT and EVENT accept removal by an existing authorized club operator, suspension of the captured author, or publishing suspension/removal of the captured parent club.
 - CHAT_MESSAGE accepts suspension of the captured sender.
-- Server-side checks verify the retained audit, target/author/club relationship, and that the action was not already reversed at resolution time.
-- Existing permissions for account, club, and publication actions remain unchanged; no administrative chat hiding, warning, or new publication-removal permission is created.
+- PROJECT accepts only an existing suspension of the captured creator.
+- CAREER_POST accepts only an existing suspension of the captured author.
+- Server-side checks verify the retained audit, target/owner relationship, temporal validity, and that the suspension was not reversed at resolution time; evidence linking serializes with reversal.
+- Existing permissions remain unchanged; no project/career removal, administrative chat hiding, warning, or new publication-removal permission is created.
 - Historical action identity remains linked if the action is reversed later.</x:v>
       </x:c>
       <x:c r="K76" s="15" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="L76" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M76" s="16"/>
       <x:c r="N76" s="16"/>
@@ -63502,9 +63505,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd2636db2bf6489e"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcf4afed417a4af2"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re673403394de4489"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c196f0c502d4659"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -65693,10 +65696,10 @@
         <x:v>Content reporting previously lacked approved target, access, lifecycle, concurrency, evidence, privacy, and notification rules.</x:v>
       </x:c>
       <x:c r="H75" s="31" t="str">
-        <x:v>Approved the bounded USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE reporting lifecycle with owner-only reporter reads and SYSTEM_ADMINISTRATION review.</x:v>
+        <x:v>Implemented the USER, CLUB, ANNOUNCEMENT, EVENT, CHAT_MESSAGE, PROJECT, and CAREER_POST reporting lifecycle with owner-only reporter reads and SYSTEM_ADMINISTRATION review.</x:v>
       </x:c>
       <x:c r="I75" s="31" t="str">
-        <x:v>Administration_Notification.drawio; One_to_One_Chat.drawio; CONTENT_REPORTING.md</x:v>
+        <x:v>Administration_Notification.drawio; One_to_One_Chat.drawio; Project_Teammate_Finder.drawio; Career_Board.drawio; CONTENT_REPORTING.md</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -65722,10 +65725,10 @@
         <x:v>The prior wording granted generic SYSTEM_ADMIN content-removal authority and referenced unavailable Project and JobPost modules.</x:v>
       </x:c>
       <x:c r="H76" s="31" t="str">
-        <x:v>Separated report resolution from action execution, retained existing action permissions, and required a verified link to qualifying committed evidence.</x:v>
+        <x:v>Separated report resolution from action execution, retained existing action permissions, and added verified owner-account suspension evidence for PROJECT and CAREER_POST without removal authority.</x:v>
       </x:c>
       <x:c r="I76" s="31" t="str">
-        <x:v>Administration_Notification.drawio; CONTENT_REPORTING.md</x:v>
+        <x:v>Administration_Notification.drawio; Project_Teammate_Finder.drawio; Career_Board.drawio; CONTENT_REPORTING.md</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -66258,7 +66261,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7597c85729464539"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R014003f93a0f4955"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66830,7 +66833,7 @@
         <x:v>Reporting</x:v>
       </x:c>
       <x:c r="C51" s="30" t="str">
-        <x:v>Supported targets are USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE. Project and career-post targets remain deferred until their modules exist.</x:v>
+        <x:v>Supported targets are USER, CLUB, ANNOUNCEMENT, EVENT, CHAT_MESSAGE, PROJECT, and CAREER_POST. Project and Career own ordinary detail access and safe immutable snapshots; accessible closed/expired content remains reportable, while missing, deleted, removed, or inaccessible targets return 404.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -66863,7 +66866,7 @@
         <x:v>Reporting</x:v>
       </x:c>
       <x:c r="C54" s="30" t="str">
-        <x:v>ACTION_TAKEN links an already committed qualifying action verified through the owning module; resolving a report never executes moderation.</x:v>
+        <x:v>ACTION_TAKEN links an already committed qualifying action verified through the owning module; resolving a report never executes moderation. PROJECT and CAREER_POST accept only an existing unreversed suspension of the captured creator/author.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -66907,13 +66910,13 @@
         <x:v>Reporting</x:v>
       </x:c>
       <x:c r="C58" s="30" t="str">
-        <x:v>Warnings, administrative chat hiding, and new publication-removal permissions are outside the bounded reporting phase.</x:v>
+        <x:v>Warnings, administrative chat hiding, new publication-removal permissions, and administrator project/career removal are outside the bounded reporting phase.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d991c7719384a72"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7672280eb674053"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66978,7 +66981,7 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="D5" s="115" t="str">
-        <x:v>The baseline includes the implemented Project Teammate Finder core lifecycle, FR_29 privacy-safe all-required-skill candidate search, and FR_30 transient weighted recommendations. Project reporting, member administration, warnings, and other deferred workflows remain outside the verified milestone.</x:v>
+        <x:v>The baseline includes the implemented Project Teammate Finder core lifecycle, FR_29 privacy-safe candidate search, FR_30 transient recommendations, Career Board, and backend content reporting for Project and Career posts. Member administration, warnings, Flutter reporting screens, and other deferred workflows remain outside the verified milestone.</x:v>
       </x:c>
       <x:c r="E5" s="116"/>
       <x:c r="F5" s="116"/>
@@ -67067,7 +67070,7 @@
         <x:v>FR_67–FR_68 — Content reporting</x:v>
       </x:c>
       <x:c r="B12" s="130" t="str">
-        <x:v>Approved bounded backend reporting for USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE with retained evidence, reviewer ownership, verified action links, reporter resolution notification, atomic history, and no action execution during resolution.</x:v>
+        <x:v>Implemented bounded backend reporting for USER, CLUB, ANNOUNCEMENT, EVENT, CHAT_MESSAGE, PROJECT, and CAREER_POST with retained evidence, reviewer ownership, verified action links, reporter resolution notification, atomic history, and no action execution during resolution. Project/Career ACTION_TAKEN evidence is limited to an unreversed suspension of the captured owner.</x:v>
       </x:c>
       <x:c r="C12" s="130"/>
       <x:c r="D12" s="130"/>
@@ -67328,7 +67331,7 @@
         <x:v>Backend complete: candidate search, transient recommendations, create/browse/detail/edit/apply/review/close/reopen/delete, memberships, audits, notifications</x:v>
       </x:c>
       <x:c r="E10" s="30" t="str">
-        <x:v>Project reporting, member leave/removal, ownership transfer, attachments, Flutter score display, and automatic chat creation remain deferred.</x:v>
+        <x:v>Project reporting is implemented. Member leave/removal, ownership transfer, attachments, Flutter score/report UI, and automatic chat creation remain deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -67342,10 +67345,10 @@
         <x:v>FR_56–FR_61, FR_81–FR_82</x:v>
       </x:c>
       <x:c r="D11" s="30" t="str">
-        <x:v>Publish, browse, save, edit and close career posts</x:v>
+        <x:v>Backend complete: publish, browse, detail, save, edit, close, retained closed/expired access, and content-report snapshot support</x:v>
       </x:c>
       <x:c r="E11" s="30" t="str">
-        <x:v>Implement after MUST modules are integrated.</x:v>
+        <x:v>Career-post reporting is implemented with captured-author suspension evidence only. Flutter screens, administrative removal, reopening, author deletion, and internal applications remain deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
@@ -67430,7 +67433,7 @@
         <x:v>Backend submission, retained evidence, administration review, verified action linking, audit, and resolution notification</x:v>
       </x:c>
       <x:c r="E16" s="30" t="str">
-        <x:v>Targets are USER, CLUB, ANNOUNCEMENT, EVENT, and CHAT_MESSAGE. Flutter screens and unavailable project/career targets remain separate.</x:v>
+        <x:v>Targets are USER, CLUB, ANNOUNCEMENT, EVENT, CHAT_MESSAGE, PROJECT, and CAREER_POST. Project/Career ACTION_TAKEN links only verified owner-account suspension. Flutter reporting screens remain separate.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" hidden="0" customHeight="1">
@@ -67467,7 +67470,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a1c775bd13c4585"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R841a103d19414817"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: clarify backend milestone scope and deferred features
</commit_message>
<xml_diff>
--- a/docs/requirements/UniConnect_Requirements_Baseline.xlsx
+++ b/docs/requirements/UniConnect_Requirements_Baseline.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="R7396c94319d84e2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Rf732b2422803441e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="Ra1685a0350ec4973"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="Rbb3dad68a9a644c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="Re89c0b7117744b83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="Rc06ba44a6d824f1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="R6285665666e546a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="R8a7c63dfc95542df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="R2cc363befd2f47d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="Reab00300cd8a446a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="R199befeab19b4c86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="R459c7c84374b486a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -32528,7 +32528,7 @@
       <x:c r="AC69" s="16"/>
       <x:c r="AD69" s="16"/>
     </x:row>
-    <x:row r="70" ht="22.5" customHeight="1">
+    <x:row r="70" ht="240" hidden="0" customHeight="1">
       <x:c r="A70" s="22" t="n">
         <x:v>69</x:v>
       </x:c>
@@ -32563,13 +32563,14 @@
 - Club results display name, category, logo, and description.
 - Results are grouped by entity type and ranked by relevance.
 - REMOVED Clubs are excluded; PUBLISHING_SUSPENDED Clubs remain visible.
-- Selecting a Club result opens the Club profile.</x:v>
+- Selecting a Club result opens the Club profile.
+- Deferred from the current backend milestone; the requirement remains in the future product baseline.</x:v>
       </x:c>
       <x:c r="K70" s="15" t="str">
         <x:v>Low</x:v>
       </x:c>
       <x:c r="L70" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deferred</x:v>
       </x:c>
       <x:c r="M70" s="16"/>
       <x:c r="N70" s="16"/>
@@ -32650,7 +32651,7 @@
       <x:c r="AC71" s="16"/>
       <x:c r="AD71" s="16"/>
     </x:row>
-    <x:row r="72" ht="22.5" customHeight="1">
+    <x:row r="72" ht="156" hidden="0" customHeight="1">
       <x:c r="A72" s="22" t="n">
         <x:v>71</x:v>
       </x:c>
@@ -32684,13 +32685,14 @@
 - AccountStatus becomes SUSPENDED.
 - Every current AuthenticatedSession is revoked in the same transaction.
 - The User immediately loses all protected platform and Club actions.
-- The state change is recorded in immutable audit history.</x:v>
+- The state change is recorded in immutable audit history.
+- Suspension has no automatic expiry or scheduled reactivation.</x:v>
       </x:c>
       <x:c r="K72" s="15" t="str">
         <x:v>Low</x:v>
       </x:c>
       <x:c r="L72" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M72" s="16"/>
       <x:c r="N72" s="16"/>
@@ -32711,7 +32713,7 @@
       <x:c r="AC72" s="16"/>
       <x:c r="AD72" s="16"/>
     </x:row>
-    <x:row r="73" ht="22.5" customHeight="1">
+    <x:row r="73" ht="144" hidden="0" customHeight="1">
       <x:c r="A73" s="22" t="n">
         <x:v>72</x:v>
       </x:c>
@@ -32744,13 +32746,14 @@
 - AccountStatus becomes ACTIVE.
 - Previously revoked AuthenticatedSessions remain revoked.
 - The member must authenticate again to create a new session.
-- The state change is recorded in immutable audit history.</x:v>
+- The state change is recorded in immutable audit history.
+- Reactivation is an explicit authorized administrator action; suspension does not expire automatically.</x:v>
       </x:c>
       <x:c r="K73" s="15" t="str">
         <x:v>Low</x:v>
       </x:c>
       <x:c r="L73" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M73" s="16"/>
       <x:c r="N73" s="16"/>
@@ -32771,7 +32774,7 @@
       <x:c r="AC73" s="16"/>
       <x:c r="AD73" s="16"/>
     </x:row>
-    <x:row r="74" ht="22.5" customHeight="1">
+    <x:row r="74" ht="252" hidden="0" customHeight="1">
       <x:c r="A74" s="22" t="n">
         <x:v>73</x:v>
       </x:c>
@@ -32807,13 +32810,14 @@
 - Login credentials and verification/reset tokens are invalidated.
 - Direct identifiers are removed or replaced with non-identifying values.
 - Historical messages, memberships, publications, moderation actions, and audit records are retained with anonymized attribution where required.
-- The account cannot log in, receive authority, or perform protected actions.</x:v>
+- The account cannot log in, receive authority, or perform protected actions.
+- Complete account anonymization is deferred; existing module privacy hooks remain future integration surfaces.</x:v>
       </x:c>
       <x:c r="K74" s="15" t="str">
         <x:v>Low</x:v>
       </x:c>
       <x:c r="L74" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Deferred</x:v>
       </x:c>
       <x:c r="M74" s="16"/>
       <x:c r="N74" s="16"/>
@@ -33278,7 +33282,7 @@
       <x:c r="AC81" s="16"/>
       <x:c r="AD81" s="16"/>
     </x:row>
-    <x:row r="82" ht="22.5" customHeight="1">
+    <x:row r="82" ht="204" hidden="0" customHeight="1">
       <x:c r="A82" s="22" t="n">
         <x:v>81</x:v>
       </x:c>
@@ -33311,13 +33315,15 @@
 - Current AccountStatus, session, context, and resource authorization are rechecked.
 - Revoked access is not restored or bypassed.
 - An unavailable or removed target produces a clear message.
-- Opening may set readAt according to configured behavior.</x:v>
+- Opening may set readAt according to configured behavior.
+- Destination APIs continue enforcing their existing access checks when clients navigate from a notification.
+- A dedicated notification-target resolution endpoint is deferred; FR_78 is not complete.</x:v>
       </x:c>
       <x:c r="K82" s="15" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="L82" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="M82" s="16"/>
       <x:c r="N82" s="16"/>
@@ -63505,9 +63511,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcf4afed417a4af2"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e8b062e2ad248ba"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c196f0c502d4659"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65850f5ab45c47c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66261,7 +66267,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R014003f93a0f4955"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82e35970afbc40de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66916,7 +66922,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7672280eb674053"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R182a87bcee8e477d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66981,7 +66987,7 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="D5" s="115" t="str">
-        <x:v>The baseline includes the implemented Project Teammate Finder core lifecycle, FR_29 privacy-safe candidate search, FR_30 transient recommendations, Career Board, and backend content reporting for Project and Career posts. Member administration, warnings, Flutter reporting screens, and other deferred workflows remain outside the verified milestone.</x:v>
+        <x:v>The approved baseline is rebuilt around one canonical User, explicit assignment-scoped Club authority, informative Events, stable direct chat, and complete agreed Project/Career backend scope including reporting. Cross-module search, complete account anonymization, and a dedicated notification-target resolution endpoint remain deferred. Suspension/reactivation remains the supported account-management flow. Frontend integration and confirmed Project/Career integration fixes remain.</x:v>
       </x:c>
       <x:c r="E5" s="116"/>
       <x:c r="F5" s="116"/>
@@ -67331,7 +67337,7 @@
         <x:v>Backend complete: candidate search, transient recommendations, create/browse/detail/edit/apply/review/close/reopen/delete, memberships, audits, notifications</x:v>
       </x:c>
       <x:c r="E10" s="30" t="str">
-        <x:v>Project reporting is implemented. Member leave/removal, ownership transfer, attachments, Flutter score/report UI, and automatic chat creation remain deferred.</x:v>
+        <x:v>Project reporting is implemented. Backend scope is complete; frontend integration and confirmed integration fixes remain. Member leave/removal, ownership transfer, attachments, and automatic chat creation remain deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -67348,7 +67354,7 @@
         <x:v>Backend complete: publish, browse, detail, save, edit, close, retained closed/expired access, and content-report snapshot support</x:v>
       </x:c>
       <x:c r="E11" s="30" t="str">
-        <x:v>Career-post reporting is implemented with captured-author suspension evidence only. Flutter screens, administrative removal, reopening, author deletion, and internal applications remain deferred.</x:v>
+        <x:v>Career-post reporting is implemented with captured-author suspension evidence only. Backend scope is complete; frontend integration and confirmed integration fixes remain. Administrative removal, reopening, author deletion, and internal applications remain deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
@@ -67362,10 +67368,10 @@
         <x:v>FR_72, FR_78</x:v>
       </x:c>
       <x:c r="D12" s="30" t="str">
-        <x:v>Informational notifications and authorized deep links</x:v>
+        <x:v>Informational notifications; destination APIs retain their own access checks</x:v>
       </x:c>
       <x:c r="E12" s="30" t="str">
-        <x:v>Start with events needed by completed modules.</x:v>
+        <x:v>A dedicated FR_78 notification-target resolution endpoint is deferred. Existing destination APIs remain authoritative; FR_78 is not complete.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="48" customHeight="1">
@@ -67379,10 +67385,10 @@
         <x:v>FR_63–FR_66, FR_68, FR_70–FR_71, FR_83</x:v>
       </x:c>
       <x:c r="D13" s="30" t="str">
-        <x:v>Account/Club moderation, anonymization and publishing restoration</x:v>
+        <x:v>Account search, suspension/reactivation, Club moderation, and publishing restoration</x:v>
       </x:c>
       <x:c r="E13" s="30" t="str">
-        <x:v>Existing account, Club, and publication actions remain authoritative; report resolution may verify their audits but never executes them.</x:v>
+        <x:v>Suspension/reactivation is the supported account-management flow. Suspension has no automatic expiry and requires explicit administrator reactivation. Complete FR_66 anonymization is deferred; existing privacy hooks remain.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="48" customHeight="1">
@@ -67390,16 +67396,16 @@
         <x:v>Cross-Module Search</x:v>
       </x:c>
       <x:c r="B14" s="30" t="str">
-        <x:v>SHOULD</x:v>
+        <x:v>DEFERRED</x:v>
       </x:c>
       <x:c r="C14" s="30" t="str">
         <x:v>FR_62</x:v>
       </x:c>
       <x:c r="D14" s="30" t="str">
-        <x:v>Search across implemented accessible content</x:v>
+        <x:v>No current milestone implementation commitment</x:v>
       </x:c>
       <x:c r="E14" s="30" t="str">
-        <x:v>Limit search to modules completed during the rebuild.</x:v>
+        <x:v>FR_62 remains in the future product baseline.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
@@ -67470,7 +67476,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R841a103d19414817"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R228a155841304b98"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: clarify backend milestone scope and deferred features (#89)
</commit_message>
<xml_diff>
--- a/docs/requirements/UniConnect_Requirements_Baseline.xlsx
+++ b/docs/requirements/UniConnect_Requirements_Baseline.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="R7396c94319d84e2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Rf732b2422803441e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="Ra1685a0350ec4973"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="Rbb3dad68a9a644c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="Re89c0b7117744b83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="Rc06ba44a6d824f1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="R6285665666e546a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="R8a7c63dfc95542df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="R2cc363befd2f47d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="Reab00300cd8a446a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="R199befeab19b4c86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="R459c7c84374b486a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -32528,7 +32528,7 @@
       <x:c r="AC69" s="16"/>
       <x:c r="AD69" s="16"/>
     </x:row>
-    <x:row r="70" ht="22.5" customHeight="1">
+    <x:row r="70" ht="240" hidden="0" customHeight="1">
       <x:c r="A70" s="22" t="n">
         <x:v>69</x:v>
       </x:c>
@@ -32563,13 +32563,14 @@
 - Club results display name, category, logo, and description.
 - Results are grouped by entity type and ranked by relevance.
 - REMOVED Clubs are excluded; PUBLISHING_SUSPENDED Clubs remain visible.
-- Selecting a Club result opens the Club profile.</x:v>
+- Selecting a Club result opens the Club profile.
+- Deferred from the current backend milestone; the requirement remains in the future product baseline.</x:v>
       </x:c>
       <x:c r="K70" s="15" t="str">
         <x:v>Low</x:v>
       </x:c>
       <x:c r="L70" s="15" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Deferred</x:v>
       </x:c>
       <x:c r="M70" s="16"/>
       <x:c r="N70" s="16"/>
@@ -32650,7 +32651,7 @@
       <x:c r="AC71" s="16"/>
       <x:c r="AD71" s="16"/>
     </x:row>
-    <x:row r="72" ht="22.5" customHeight="1">
+    <x:row r="72" ht="156" hidden="0" customHeight="1">
       <x:c r="A72" s="22" t="n">
         <x:v>71</x:v>
       </x:c>
@@ -32684,13 +32685,14 @@
 - AccountStatus becomes SUSPENDED.
 - Every current AuthenticatedSession is revoked in the same transaction.
 - The User immediately loses all protected platform and Club actions.
-- The state change is recorded in immutable audit history.</x:v>
+- The state change is recorded in immutable audit history.
+- Suspension has no automatic expiry or scheduled reactivation.</x:v>
       </x:c>
       <x:c r="K72" s="15" t="str">
         <x:v>Low</x:v>
       </x:c>
       <x:c r="L72" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M72" s="16"/>
       <x:c r="N72" s="16"/>
@@ -32711,7 +32713,7 @@
       <x:c r="AC72" s="16"/>
       <x:c r="AD72" s="16"/>
     </x:row>
-    <x:row r="73" ht="22.5" customHeight="1">
+    <x:row r="73" ht="144" hidden="0" customHeight="1">
       <x:c r="A73" s="22" t="n">
         <x:v>72</x:v>
       </x:c>
@@ -32744,13 +32746,14 @@
 - AccountStatus becomes ACTIVE.
 - Previously revoked AuthenticatedSessions remain revoked.
 - The member must authenticate again to create a new session.
-- The state change is recorded in immutable audit history.</x:v>
+- The state change is recorded in immutable audit history.
+- Reactivation is an explicit authorized administrator action; suspension does not expire automatically.</x:v>
       </x:c>
       <x:c r="K73" s="15" t="str">
         <x:v>Low</x:v>
       </x:c>
       <x:c r="L73" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M73" s="16"/>
       <x:c r="N73" s="16"/>
@@ -32771,7 +32774,7 @@
       <x:c r="AC73" s="16"/>
       <x:c r="AD73" s="16"/>
     </x:row>
-    <x:row r="74" ht="22.5" customHeight="1">
+    <x:row r="74" ht="252" hidden="0" customHeight="1">
       <x:c r="A74" s="22" t="n">
         <x:v>73</x:v>
       </x:c>
@@ -32807,13 +32810,14 @@
 - Login credentials and verification/reset tokens are invalidated.
 - Direct identifiers are removed or replaced with non-identifying values.
 - Historical messages, memberships, publications, moderation actions, and audit records are retained with anonymized attribution where required.
-- The account cannot log in, receive authority, or perform protected actions.</x:v>
+- The account cannot log in, receive authority, or perform protected actions.
+- Complete account anonymization is deferred; existing module privacy hooks remain future integration surfaces.</x:v>
       </x:c>
       <x:c r="K74" s="15" t="str">
         <x:v>Low</x:v>
       </x:c>
       <x:c r="L74" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>Deferred</x:v>
       </x:c>
       <x:c r="M74" s="16"/>
       <x:c r="N74" s="16"/>
@@ -33278,7 +33282,7 @@
       <x:c r="AC81" s="16"/>
       <x:c r="AD81" s="16"/>
     </x:row>
-    <x:row r="82" ht="22.5" customHeight="1">
+    <x:row r="82" ht="204" hidden="0" customHeight="1">
       <x:c r="A82" s="22" t="n">
         <x:v>81</x:v>
       </x:c>
@@ -33311,13 +33315,15 @@
 - Current AccountStatus, session, context, and resource authorization are rechecked.
 - Revoked access is not restored or bypassed.
 - An unavailable or removed target produces a clear message.
-- Opening may set readAt according to configured behavior.</x:v>
+- Opening may set readAt according to configured behavior.
+- Destination APIs continue enforcing their existing access checks when clients navigate from a notification.
+- A dedicated notification-target resolution endpoint is deferred; FR_78 is not complete.</x:v>
       </x:c>
       <x:c r="K82" s="15" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="L82" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="M82" s="16"/>
       <x:c r="N82" s="16"/>
@@ -63505,9 +63511,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcf4afed417a4af2"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e8b062e2ad248ba"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c196f0c502d4659"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65850f5ab45c47c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66261,7 +66267,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R014003f93a0f4955"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82e35970afbc40de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66916,7 +66922,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7672280eb674053"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R182a87bcee8e477d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66981,7 +66987,7 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="D5" s="115" t="str">
-        <x:v>The baseline includes the implemented Project Teammate Finder core lifecycle, FR_29 privacy-safe candidate search, FR_30 transient recommendations, Career Board, and backend content reporting for Project and Career posts. Member administration, warnings, Flutter reporting screens, and other deferred workflows remain outside the verified milestone.</x:v>
+        <x:v>The approved baseline is rebuilt around one canonical User, explicit assignment-scoped Club authority, informative Events, stable direct chat, and complete agreed Project/Career backend scope including reporting. Cross-module search, complete account anonymization, and a dedicated notification-target resolution endpoint remain deferred. Suspension/reactivation remains the supported account-management flow. Frontend integration and confirmed Project/Career integration fixes remain.</x:v>
       </x:c>
       <x:c r="E5" s="116"/>
       <x:c r="F5" s="116"/>
@@ -67331,7 +67337,7 @@
         <x:v>Backend complete: candidate search, transient recommendations, create/browse/detail/edit/apply/review/close/reopen/delete, memberships, audits, notifications</x:v>
       </x:c>
       <x:c r="E10" s="30" t="str">
-        <x:v>Project reporting is implemented. Member leave/removal, ownership transfer, attachments, Flutter score/report UI, and automatic chat creation remain deferred.</x:v>
+        <x:v>Project reporting is implemented. Backend scope is complete; frontend integration and confirmed integration fixes remain. Member leave/removal, ownership transfer, attachments, and automatic chat creation remain deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -67348,7 +67354,7 @@
         <x:v>Backend complete: publish, browse, detail, save, edit, close, retained closed/expired access, and content-report snapshot support</x:v>
       </x:c>
       <x:c r="E11" s="30" t="str">
-        <x:v>Career-post reporting is implemented with captured-author suspension evidence only. Flutter screens, administrative removal, reopening, author deletion, and internal applications remain deferred.</x:v>
+        <x:v>Career-post reporting is implemented with captured-author suspension evidence only. Backend scope is complete; frontend integration and confirmed integration fixes remain. Administrative removal, reopening, author deletion, and internal applications remain deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
@@ -67362,10 +67368,10 @@
         <x:v>FR_72, FR_78</x:v>
       </x:c>
       <x:c r="D12" s="30" t="str">
-        <x:v>Informational notifications and authorized deep links</x:v>
+        <x:v>Informational notifications; destination APIs retain their own access checks</x:v>
       </x:c>
       <x:c r="E12" s="30" t="str">
-        <x:v>Start with events needed by completed modules.</x:v>
+        <x:v>A dedicated FR_78 notification-target resolution endpoint is deferred. Existing destination APIs remain authoritative; FR_78 is not complete.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="48" customHeight="1">
@@ -67379,10 +67385,10 @@
         <x:v>FR_63–FR_66, FR_68, FR_70–FR_71, FR_83</x:v>
       </x:c>
       <x:c r="D13" s="30" t="str">
-        <x:v>Account/Club moderation, anonymization and publishing restoration</x:v>
+        <x:v>Account search, suspension/reactivation, Club moderation, and publishing restoration</x:v>
       </x:c>
       <x:c r="E13" s="30" t="str">
-        <x:v>Existing account, Club, and publication actions remain authoritative; report resolution may verify their audits but never executes them.</x:v>
+        <x:v>Suspension/reactivation is the supported account-management flow. Suspension has no automatic expiry and requires explicit administrator reactivation. Complete FR_66 anonymization is deferred; existing privacy hooks remain.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="48" customHeight="1">
@@ -67390,16 +67396,16 @@
         <x:v>Cross-Module Search</x:v>
       </x:c>
       <x:c r="B14" s="30" t="str">
-        <x:v>SHOULD</x:v>
+        <x:v>DEFERRED</x:v>
       </x:c>
       <x:c r="C14" s="30" t="str">
         <x:v>FR_62</x:v>
       </x:c>
       <x:c r="D14" s="30" t="str">
-        <x:v>Search across implemented accessible content</x:v>
+        <x:v>No current milestone implementation commitment</x:v>
       </x:c>
       <x:c r="E14" s="30" t="str">
-        <x:v>Limit search to modules completed during the rebuild.</x:v>
+        <x:v>FR_62 remains in the future product baseline.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
@@ -67470,7 +67476,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R841a103d19414817"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R228a155841304b98"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(mentorship): correct scheduling and enrollment lifecycle (#90)
</commit_message>
<xml_diff>
--- a/docs/requirements/UniConnect_Requirements_Baseline.xlsx
+++ b/docs/requirements/UniConnect_Requirements_Baseline.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="R6285665666e546a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="R8a7c63dfc95542df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="R2cc363befd2f47d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="Reab00300cd8a446a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="R199befeab19b4c86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="R459c7c84374b486a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="R90e851546b304908"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Rbc348300cf93413d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="R5839b82f7271451e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="R873682e8d0f94330"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="R5ebaacc48b9e4c15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="Rd3dc258213a0452a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -31326,7 +31326,7 @@
         <x:v>FR_42</x:v>
       </x:c>
       <x:c r="C50" s="13" t="str">
-        <x:v>The system shall allow a registered Mentor to create a ONE_TIME, WEEKLY, or BIWEEKLY MentorshipSlot series and its dated occurrences.</x:v>
+        <x:v>The system shall allow a registered Mentor to create a finite ONE_TIME, WEEKLY, or BIWEEKLY MentorshipSlot series with authoritative dated occurrences.</x:v>
       </x:c>
       <x:c r="D50" s="12" t="str">
         <x:v>US_42</x:v>
@@ -31348,18 +31348,18 @@
       </x:c>
       <x:c r="J50" s="13" t="str">
         <x:v>- Topic, description, schedule type, start/end times, mode, and capacity are required.
-- End time is later than start time.
-- ONE_TIME creates exactly one dated occurrence.
-- WEEKLY and BIWEEKLY require a recurrence end date and generate dated future occurrences.
-- IN_PERSON requires a location; ONLINE requires a meeting link.
-- Conflicting mentor schedules are rejected.
-- A valid slot is created with SlotStatus = OPEN.</x:v>
+- Schedule dates and times use Asia/Dhaka; lifecycle timestamps use UTC.
+- ONE_TIME creates exactly one occurrence; recurring series use an end date or fixed meeting count.
+- A series contains at most 52 meetings; an omitted legacy/client bound retains the established 12-meeting behavior.
+- Authoritative dated occurrences are persisted without silently truncating a requested valid schedule.
+- Every proposed occurrence is checked against the mentor's uncancelled hosted occurrences with [start, end) overlap semantics.
+- A valid series opens enrollment independently of derived fullness.</x:v>
       </x:c>
       <x:c r="K50" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L50" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="M50" s="16"/>
       <x:c r="N50" s="16"/>
@@ -31509,7 +31509,7 @@
         <x:v>FR_45</x:v>
       </x:c>
       <x:c r="C53" s="13" t="str">
-        <x:v>The system shall allow an ACTIVE Student to enroll once in an OPEN MentorshipSlot series with available capacity.</x:v>
+        <x:v>The system shall allow an ACTIVE, non-anonymized Student or Alumni user to enroll in another mentor's open MentorshipSlot series while a future meeting and capacity remain.</x:v>
       </x:c>
       <x:c r="D53" s="12" t="str">
         <x:v>US_45</x:v>
@@ -31518,30 +31518,31 @@
         <x:v>Reserve a Mentorship Place</x:v>
       </x:c>
       <x:c r="F53" s="19" t="str">
-        <x:v>Student</x:v>
+        <x:v>Active Student or Alumni</x:v>
       </x:c>
       <x:c r="G53" s="19" t="str">
-        <x:v>to join an open mentorship slot with available capacity</x:v>
+        <x:v>to join another mentor's open series with available capacity</x:v>
       </x:c>
       <x:c r="H53" s="19" t="str">
-        <x:v>I can receive mentorship from experienced individuals</x:v>
+        <x:v>I can participate in the remaining meetings without losing earlier history</x:v>
       </x:c>
       <x:c r="I53" s="13" t="str">
-        <x:v>As a Student, I want to join an open mentorship slot with available capacity, so that I can receive mentorship from experienced individuals.</x:v>
+        <x:v>As an active Student or Alumni, I want to join another mentor's open mentorship series so that I can participate in its remaining meetings.</x:v>
       </x:c>
       <x:c r="J53" s="13" t="str">
-        <x:v>- The mentee has PlatformRole = STUDENT and AccountStatus = ACTIVE.
-- The slot is OPEN, has a future uncancelled occurrence, and has derived available capacity.
-- The creating Mentor cannot join their own slot.
-- At most one current enrollment exists per slot/student pair.
-- One enrollment covers the complete slot series.
-- The derived enrollment count reflects the new enrollment and confirmation notifications are generated.</x:v>
+        <x:v>- PlatformRole is STUDENT or ALUMNI; AccountStatus is ACTIVE and the account is not anonymized.
+- Mentors may enroll in another mentor's series but never their own.
+- Enrollment is open, the mentor is AVAILABLE, capacity remains, and an uncancelled meeting that has not started exists.
+- The applicant is rejected only when a future series meeting overlaps a meeting they host; meetings they merely attend do not block enrollment.
+- One active enrollment exists per user/series and concurrent final-place requests cannot overbook.
+- Joining midway covers only meetings that have not started; one enrollment covers all remaining meetings.
+- Derived count, vacancy, and fullness update atomically and notifications are emitted once.</x:v>
       </x:c>
       <x:c r="K53" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L53" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="M53" s="16"/>
       <x:c r="N53" s="16"/>
@@ -31570,7 +31571,7 @@
         <x:v>FR_46</x:v>
       </x:c>
       <x:c r="C54" s="13" t="str">
-        <x:v>The system shall allow an enrolled Student to leave a mentorship slot.</x:v>
+        <x:v>The system shall allow an enrolled Student or Alumni to leave and later rejoin an eligible mentorship series while preserving every participation period.</x:v>
       </x:c>
       <x:c r="D54" s="12" t="str">
         <x:v>US_46</x:v>
@@ -31579,30 +31580,29 @@
         <x:v>Release My Mentorship Place</x:v>
       </x:c>
       <x:c r="F54" s="19" t="str">
-        <x:v>enrolled Student</x:v>
+        <x:v>enrolled Student or Alumni</x:v>
       </x:c>
       <x:c r="G54" s="19" t="str">
-        <x:v>to leave a mentorship slot</x:v>
+        <x:v>to leave and later rejoin an eligible mentorship series</x:v>
       </x:c>
       <x:c r="H54" s="19" t="str">
-        <x:v>I can free up my schedule and allow others to take the spot if my circumstances change</x:v>
+        <x:v>I can release capacity without losing participation history</x:v>
       </x:c>
       <x:c r="I54" s="13" t="str">
-        <x:v>As an enrolled Student, I want to leave a mentorship slot, so that I can free up my schedule and allow others to take the spot if my circumstances change.</x:v>
+        <x:v>As an enrolled Student or Alumni, I want to leave and later rejoin an eligible mentorship series so that capacity and my participation history remain accurate.</x:v>
       </x:c>
       <x:c r="J54" s="13" t="str">
-        <x:v>- Only a currently enrolled Student may leave.
-- Confirmation is required.
-- Leaving sets leftAt and preserves enrollment history.
-- The derived enrollment and available-place counts update.
-- A previously FULL slot is no longer labelled FULL when capacity becomes available.
-- Existing occurrence history is preserved.</x:v>
+        <x:v>- Only a current enrollment may transition to LEFT; an identical retry creates no second transition or notification.
+- Leaving records the period's leftAt, frees derived capacity, and removes meeting-link access.
+- Rejoining is allowed only under the normal availability, vacancy, future-meeting, and hosted-conflict checks.
+- Rejoining creates a new participation period and never overwrites earlier join/leave timestamps or private notes.
+- Existing occurrence and enrollment history is preserved.</x:v>
       </x:c>
       <x:c r="K54" s="15" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="L54" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="M54" s="16"/>
       <x:c r="N54" s="16"/>
@@ -31652,18 +31652,18 @@
         <x:v>As a Mentorship Slot Creator, I want to update the permitted details of my mentorship slot, so that I can keep the mentorship information accurate and up-to-date.</x:v>
       </x:c>
       <x:c r="J55" s="13" t="str">
-        <x:v>- Only the MentorProfile owner may edit.
-- Schedule changes are checked for conflicts.
-- Capacity cannot be lower than the current derived enrollment count.
-- Past occurrences are preserved.
-- Recurring-series changes affect only eligible future occurrences.
-- Current mentees are notified of material changes.</x:v>
+        <x:v>- Only the hosting MentorProfile owner may edit.
+- Past and ongoing occurrences are preserved; only meetings that have not started are replaced.
+- Every proposed future occurrence is checked only against the host mentor's uncancelled hosted schedule using [start, end) overlap semantics.
+- Enrolled mentees' hosting commitments do not block the edit.
+- Capacity may increase or decrease but never below authoritative active enrollment.
+- Current mentees are notified once only when relevant details materially change.</x:v>
       </x:c>
       <x:c r="K55" s="15" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="L55" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="M55" s="16"/>
       <x:c r="N55" s="16"/>
@@ -31713,17 +31713,18 @@
         <x:v>As the creator of a mentorship slot, I want to stop accepting new mentees, so that I can manage my capacity and focus on existing mentees.</x:v>
       </x:c>
       <x:c r="J56" s="13" t="str">
-        <x:v>- Only creator can close.
-- Status becomes Closed.
-- Existing mentees remain enrolled.
-- New joins are rejected.
-- Closed status is visible.</x:v>
+        <x:v>- Only the hosting mentor may close or reopen enrollment.
+- Closing blocks joins and rejoins but preserves current enrollments and all meetings.
+- Closing is independent of derived FULL and does not complete the series.
+- Reopening requires a future meeting and vacancy; a cancelled series cannot reopen.
+- Mentor availability changes do not erase explicit closure.
+- Identical lifecycle retries create no duplicate transition or notification.</x:v>
       </x:c>
       <x:c r="K56" s="15" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="L56" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="M56" s="16"/>
       <x:c r="N56" s="16"/>
@@ -31773,17 +31774,17 @@
         <x:v>As the creator of a mentorship slot, I want to cancel the slot when I can no  longer conduct a session and notify its enrolled mentees, so that they are informed in advance and can make alternative arrangements.</x:v>
       </x:c>
       <x:c r="J57" s="13" t="str">
-        <x:v>- Only the MentorProfile owner may cancel.
-- Confirmation is required.
-- SlotStatus becomes CANCELLED and new enrollments are blocked.
-- Current enrollments and past occurrence history are preserved.
-- Every currently enrolled mentee receives one cancellation notification event.</x:v>
+        <x:v>- Only the hosting mentor may cancel.
+- Cancellation blocks enrollment and cancels meetings that have not started; past and ongoing occurrences remain unchanged.
+- Current participation and occurrence history are retained.
+- Every current mentee receives one cancellation notification event.
+- An identical cancellation retry creates no duplicate transition or notification.</x:v>
       </x:c>
       <x:c r="K57" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L57" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="M57" s="16"/>
       <x:c r="N57" s="16"/>
@@ -31812,7 +31813,7 @@
         <x:v>FR_50</x:v>
       </x:c>
       <x:c r="C58" s="13" t="str">
-        <x:v>The system shall allow a mentor or enrolled Student to view MentorshipSlot series they created or joined.</x:v>
+        <x:v>The system shall allow a hosting mentor or participating Student or Alumni to view authorized current and historical MentorshipSlot participation.</x:v>
       </x:c>
       <x:c r="D58" s="12" t="str">
         <x:v>US_50</x:v>
@@ -31821,30 +31822,30 @@
         <x:v>Track My Joined Mentorship Sessions</x:v>
       </x:c>
       <x:c r="F58" s="19" t="str">
-        <x:v>Mentor or enrolled Student</x:v>
+        <x:v>hosting mentor or participating member</x:v>
       </x:c>
       <x:c r="G58" s="19" t="str">
-        <x:v>to view the mentorship slots I created or joined</x:v>
+        <x:v>to view mentorship series I host or participation periods I joined</x:v>
       </x:c>
       <x:c r="H58" s="19" t="str">
-        <x:v>I can track my mentoring activities and commitments</x:v>
+        <x:v>I can distinguish ongoing, next, completed, left, and cancelled activity</x:v>
       </x:c>
       <x:c r="I58" s="13" t="str">
-        <x:v>As a Student, I want to view the mentorship slots I created or joined, so that I can track my mentoring activities and commitments.</x:v>
+        <x:v>As a mentorship participant, I want authorized current and historical views so that I can track my activities and commitments.</x:v>
       </x:c>
       <x:c r="J58" s="13" t="str">
-        <x:v>- Student and Alumni mentors see slot series they created.
-- Student mentees see slot series they joined.
-- The next eligible occurrence date/time is shown.
-- Location or meeting link is shown according to mode.
-- Stored slot status and derived FULL/past labels are shown.
-- Historical left, cancelled, and past records remain available where authorized.</x:v>
+        <x:v>- Student and Alumni mentors see series they host; each participant sees their own participation periods and private join message/goals.
+- Ongoing occurrence and the next meeting that has not started are distinct fields.
+- Completed, left, and cancelled periods remain in authorized history; closure does not imply completion.
+- Only the host may retrieve the roster.
+- Meeting links appear only to the host and currently enrolled participants with a remaining ongoing or future meeting.
+- Leaving or historical participation alone cannot reveal the link on detail, list, history, or occurrence-related responses.</x:v>
       </x:c>
       <x:c r="K58" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L58" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="M58" s="16"/>
       <x:c r="N58" s="16"/>
@@ -63511,9 +63512,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e8b062e2ad248ba"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9989f435867f4f3c"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65850f5ab45c47c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48ae02b4428c43dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66267,7 +66268,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82e35970afbc40de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reafa9bc430ab4583"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66608,7 +66609,7 @@
         <x:v>Mentorship</x:v>
       </x:c>
       <x:c r="C30" s="31" t="str">
-        <x:v>MentorshipSlot supports ONE_TIME, WEEKLY, and BIWEEKLY series with dated MentorshipOccurrences.</x:v>
+        <x:v>ACTIVE, non-anonymized Year-2-or-above Students and ACTIVE, non-anonymized Alumni may register as mentors; mentor availability controls new enrollment, not existing series.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -66619,7 +66620,7 @@
         <x:v>Mentorship</x:v>
       </x:c>
       <x:c r="C31" s="31" t="str">
-        <x:v>One MentorshipEnrollment enrolls an ACTIVE STUDENT in the complete series.</x:v>
+        <x:v>MentorshipSlot supports finite ONE_TIME, WEEKLY, and BIWEEKLY schedules. Asia/Dhaka schedule values generate authoritative dated MentorshipOccurrences; past and ongoing occurrences survive future-only edits and cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -66630,7 +66631,7 @@
         <x:v>Mentorship</x:v>
       </x:c>
       <x:c r="C32" s="31" t="str">
-        <x:v>Enrollment count, available places, FULL, and past state are derived; historical records are retained.</x:v>
+        <x:v>One active enrollment covers a series' remaining unstarted meetings for an ACTIVE Student or Alumni. Other mentors may enroll, self-enrollment is forbidden, hosted-meeting conflicts block join, and leave/rejoin creates separate retained participation periods.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -66641,7 +66642,7 @@
         <x:v>Career</x:v>
       </x:c>
       <x:c r="C33" s="31" t="str">
-        <x:v>Only ACTIVE ALUMNI users publish JobPosts; no separate alumni-verification state exists.</x:v>
+        <x:v>Enrollment closure, mentor availability, derived FULL, completion, and cancellation are distinct. Counts and vacancies derive from active enrollment; only hosts see rosters, and meeting links are limited to hosts and current participants with a remaining meeting.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -66922,7 +66923,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R182a87bcee8e477d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d62dea8aa394740"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -67413,16 +67414,16 @@
         <x:v>Peer Mentorship</x:v>
       </x:c>
       <x:c r="B15" s="30" t="str">
-        <x:v>DEFERRED</x:v>
+        <x:v>SHOULD</x:v>
       </x:c>
       <x:c r="C15" s="30" t="str">
         <x:v>FR_40–FR_50</x:v>
       </x:c>
       <x:c r="D15" s="30" t="str">
-        <x:v>No one-month commitment</x:v>
+        <x:v>Backend lifecycle corrections in progress: finite occurrences, enrollment periods, conflict/capacity serialization, privacy-safe responses, and retained history</x:v>
       </x:c>
       <x:c r="E15" s="30" t="str">
-        <x:v>Retained in the product baseline for later implementation.</x:v>
+        <x:v>Flutter remains on existing endpoint shapes where practical. Reopen and history fields/endpoints are additive; cross-module search, complete anonymization, and the dedicated notification-target resolver remain deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="36" hidden="0" customHeight="1">
@@ -67476,7 +67477,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R228a155841304b98"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffb473c9d31a458a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(mentorship): correct scheduling and enrollment lifecycle (#90) (#91)
</commit_message>
<xml_diff>
--- a/docs/requirements/UniConnect_Requirements_Baseline.xlsx
+++ b/docs/requirements/UniConnect_Requirements_Baseline.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="R6285665666e546a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="R8a7c63dfc95542df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="R2cc363befd2f47d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="Reab00300cd8a446a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="R199befeab19b4c86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="R459c7c84374b486a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Info" sheetId="1" r:id="R90e851546b304908"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FR, User Stories" sheetId="2" r:id="Rbc348300cf93413d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Audit" sheetId="3" r:id="R5839b82f7271451e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confirmed Rules" sheetId="4" r:id="R873682e8d0f94330"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Summary" sheetId="5" r:id="R5ebaacc48b9e4c15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Implementation Scope" sheetId="6" r:id="Rd3dc258213a0452a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -31326,7 +31326,7 @@
         <x:v>FR_42</x:v>
       </x:c>
       <x:c r="C50" s="13" t="str">
-        <x:v>The system shall allow a registered Mentor to create a ONE_TIME, WEEKLY, or BIWEEKLY MentorshipSlot series and its dated occurrences.</x:v>
+        <x:v>The system shall allow a registered Mentor to create a finite ONE_TIME, WEEKLY, or BIWEEKLY MentorshipSlot series with authoritative dated occurrences.</x:v>
       </x:c>
       <x:c r="D50" s="12" t="str">
         <x:v>US_42</x:v>
@@ -31348,18 +31348,18 @@
       </x:c>
       <x:c r="J50" s="13" t="str">
         <x:v>- Topic, description, schedule type, start/end times, mode, and capacity are required.
-- End time is later than start time.
-- ONE_TIME creates exactly one dated occurrence.
-- WEEKLY and BIWEEKLY require a recurrence end date and generate dated future occurrences.
-- IN_PERSON requires a location; ONLINE requires a meeting link.
-- Conflicting mentor schedules are rejected.
-- A valid slot is created with SlotStatus = OPEN.</x:v>
+- Schedule dates and times use Asia/Dhaka; lifecycle timestamps use UTC.
+- ONE_TIME creates exactly one occurrence; recurring series use an end date or fixed meeting count.
+- A series contains at most 52 meetings; an omitted legacy/client bound retains the established 12-meeting behavior.
+- Authoritative dated occurrences are persisted without silently truncating a requested valid schedule.
+- Every proposed occurrence is checked against the mentor's uncancelled hosted occurrences with [start, end) overlap semantics.
+- A valid series opens enrollment independently of derived fullness.</x:v>
       </x:c>
       <x:c r="K50" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L50" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="M50" s="16"/>
       <x:c r="N50" s="16"/>
@@ -31509,7 +31509,7 @@
         <x:v>FR_45</x:v>
       </x:c>
       <x:c r="C53" s="13" t="str">
-        <x:v>The system shall allow an ACTIVE Student to enroll once in an OPEN MentorshipSlot series with available capacity.</x:v>
+        <x:v>The system shall allow an ACTIVE, non-anonymized Student or Alumni user to enroll in another mentor's open MentorshipSlot series while a future meeting and capacity remain.</x:v>
       </x:c>
       <x:c r="D53" s="12" t="str">
         <x:v>US_45</x:v>
@@ -31518,30 +31518,31 @@
         <x:v>Reserve a Mentorship Place</x:v>
       </x:c>
       <x:c r="F53" s="19" t="str">
-        <x:v>Student</x:v>
+        <x:v>Active Student or Alumni</x:v>
       </x:c>
       <x:c r="G53" s="19" t="str">
-        <x:v>to join an open mentorship slot with available capacity</x:v>
+        <x:v>to join another mentor's open series with available capacity</x:v>
       </x:c>
       <x:c r="H53" s="19" t="str">
-        <x:v>I can receive mentorship from experienced individuals</x:v>
+        <x:v>I can participate in the remaining meetings without losing earlier history</x:v>
       </x:c>
       <x:c r="I53" s="13" t="str">
-        <x:v>As a Student, I want to join an open mentorship slot with available capacity, so that I can receive mentorship from experienced individuals.</x:v>
+        <x:v>As an active Student or Alumni, I want to join another mentor's open mentorship series so that I can participate in its remaining meetings.</x:v>
       </x:c>
       <x:c r="J53" s="13" t="str">
-        <x:v>- The mentee has PlatformRole = STUDENT and AccountStatus = ACTIVE.
-- The slot is OPEN, has a future uncancelled occurrence, and has derived available capacity.
-- The creating Mentor cannot join their own slot.
-- At most one current enrollment exists per slot/student pair.
-- One enrollment covers the complete slot series.
-- The derived enrollment count reflects the new enrollment and confirmation notifications are generated.</x:v>
+        <x:v>- PlatformRole is STUDENT or ALUMNI; AccountStatus is ACTIVE and the account is not anonymized.
+- Mentors may enroll in another mentor's series but never their own.
+- Enrollment is open, the mentor is AVAILABLE, capacity remains, and an uncancelled meeting that has not started exists.
+- The applicant is rejected only when a future series meeting overlaps a meeting they host; meetings they merely attend do not block enrollment.
+- One active enrollment exists per user/series and concurrent final-place requests cannot overbook.
+- Joining midway covers only meetings that have not started; one enrollment covers all remaining meetings.
+- Derived count, vacancy, and fullness update atomically and notifications are emitted once.</x:v>
       </x:c>
       <x:c r="K53" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L53" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="M53" s="16"/>
       <x:c r="N53" s="16"/>
@@ -31570,7 +31571,7 @@
         <x:v>FR_46</x:v>
       </x:c>
       <x:c r="C54" s="13" t="str">
-        <x:v>The system shall allow an enrolled Student to leave a mentorship slot.</x:v>
+        <x:v>The system shall allow an enrolled Student or Alumni to leave and later rejoin an eligible mentorship series while preserving every participation period.</x:v>
       </x:c>
       <x:c r="D54" s="12" t="str">
         <x:v>US_46</x:v>
@@ -31579,30 +31580,29 @@
         <x:v>Release My Mentorship Place</x:v>
       </x:c>
       <x:c r="F54" s="19" t="str">
-        <x:v>enrolled Student</x:v>
+        <x:v>enrolled Student or Alumni</x:v>
       </x:c>
       <x:c r="G54" s="19" t="str">
-        <x:v>to leave a mentorship slot</x:v>
+        <x:v>to leave and later rejoin an eligible mentorship series</x:v>
       </x:c>
       <x:c r="H54" s="19" t="str">
-        <x:v>I can free up my schedule and allow others to take the spot if my circumstances change</x:v>
+        <x:v>I can release capacity without losing participation history</x:v>
       </x:c>
       <x:c r="I54" s="13" t="str">
-        <x:v>As an enrolled Student, I want to leave a mentorship slot, so that I can free up my schedule and allow others to take the spot if my circumstances change.</x:v>
+        <x:v>As an enrolled Student or Alumni, I want to leave and later rejoin an eligible mentorship series so that capacity and my participation history remain accurate.</x:v>
       </x:c>
       <x:c r="J54" s="13" t="str">
-        <x:v>- Only a currently enrolled Student may leave.
-- Confirmation is required.
-- Leaving sets leftAt and preserves enrollment history.
-- The derived enrollment and available-place counts update.
-- A previously FULL slot is no longer labelled FULL when capacity becomes available.
-- Existing occurrence history is preserved.</x:v>
+        <x:v>- Only a current enrollment may transition to LEFT; an identical retry creates no second transition or notification.
+- Leaving records the period's leftAt, frees derived capacity, and removes meeting-link access.
+- Rejoining is allowed only under the normal availability, vacancy, future-meeting, and hosted-conflict checks.
+- Rejoining creates a new participation period and never overwrites earlier join/leave timestamps or private notes.
+- Existing occurrence and enrollment history is preserved.</x:v>
       </x:c>
       <x:c r="K54" s="15" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="L54" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="M54" s="16"/>
       <x:c r="N54" s="16"/>
@@ -31652,18 +31652,18 @@
         <x:v>As a Mentorship Slot Creator, I want to update the permitted details of my mentorship slot, so that I can keep the mentorship information accurate and up-to-date.</x:v>
       </x:c>
       <x:c r="J55" s="13" t="str">
-        <x:v>- Only the MentorProfile owner may edit.
-- Schedule changes are checked for conflicts.
-- Capacity cannot be lower than the current derived enrollment count.
-- Past occurrences are preserved.
-- Recurring-series changes affect only eligible future occurrences.
-- Current mentees are notified of material changes.</x:v>
+        <x:v>- Only the hosting MentorProfile owner may edit.
+- Past and ongoing occurrences are preserved; only meetings that have not started are replaced.
+- Every proposed future occurrence is checked only against the host mentor's uncancelled hosted schedule using [start, end) overlap semantics.
+- Enrolled mentees' hosting commitments do not block the edit.
+- Capacity may increase or decrease but never below authoritative active enrollment.
+- Current mentees are notified once only when relevant details materially change.</x:v>
       </x:c>
       <x:c r="K55" s="15" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="L55" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="M55" s="16"/>
       <x:c r="N55" s="16"/>
@@ -31713,17 +31713,18 @@
         <x:v>As the creator of a mentorship slot, I want to stop accepting new mentees, so that I can manage my capacity and focus on existing mentees.</x:v>
       </x:c>
       <x:c r="J56" s="13" t="str">
-        <x:v>- Only creator can close.
-- Status becomes Closed.
-- Existing mentees remain enrolled.
-- New joins are rejected.
-- Closed status is visible.</x:v>
+        <x:v>- Only the hosting mentor may close or reopen enrollment.
+- Closing blocks joins and rejoins but preserves current enrollments and all meetings.
+- Closing is independent of derived FULL and does not complete the series.
+- Reopening requires a future meeting and vacancy; a cancelled series cannot reopen.
+- Mentor availability changes do not erase explicit closure.
+- Identical lifecycle retries create no duplicate transition or notification.</x:v>
       </x:c>
       <x:c r="K56" s="15" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="L56" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="M56" s="16"/>
       <x:c r="N56" s="16"/>
@@ -31773,17 +31774,17 @@
         <x:v>As the creator of a mentorship slot, I want to cancel the slot when I can no  longer conduct a session and notify its enrolled mentees, so that they are informed in advance and can make alternative arrangements.</x:v>
       </x:c>
       <x:c r="J57" s="13" t="str">
-        <x:v>- Only the MentorProfile owner may cancel.
-- Confirmation is required.
-- SlotStatus becomes CANCELLED and new enrollments are blocked.
-- Current enrollments and past occurrence history are preserved.
-- Every currently enrolled mentee receives one cancellation notification event.</x:v>
+        <x:v>- Only the hosting mentor may cancel.
+- Cancellation blocks enrollment and cancels meetings that have not started; past and ongoing occurrences remain unchanged.
+- Current participation and occurrence history are retained.
+- Every current mentee receives one cancellation notification event.
+- An identical cancellation retry creates no duplicate transition or notification.</x:v>
       </x:c>
       <x:c r="K57" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L57" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="M57" s="16"/>
       <x:c r="N57" s="16"/>
@@ -31812,7 +31813,7 @@
         <x:v>FR_50</x:v>
       </x:c>
       <x:c r="C58" s="13" t="str">
-        <x:v>The system shall allow a mentor or enrolled Student to view MentorshipSlot series they created or joined.</x:v>
+        <x:v>The system shall allow a hosting mentor or participating Student or Alumni to view authorized current and historical MentorshipSlot participation.</x:v>
       </x:c>
       <x:c r="D58" s="12" t="str">
         <x:v>US_50</x:v>
@@ -31821,30 +31822,30 @@
         <x:v>Track My Joined Mentorship Sessions</x:v>
       </x:c>
       <x:c r="F58" s="19" t="str">
-        <x:v>Mentor or enrolled Student</x:v>
+        <x:v>hosting mentor or participating member</x:v>
       </x:c>
       <x:c r="G58" s="19" t="str">
-        <x:v>to view the mentorship slots I created or joined</x:v>
+        <x:v>to view mentorship series I host or participation periods I joined</x:v>
       </x:c>
       <x:c r="H58" s="19" t="str">
-        <x:v>I can track my mentoring activities and commitments</x:v>
+        <x:v>I can distinguish ongoing, next, completed, left, and cancelled activity</x:v>
       </x:c>
       <x:c r="I58" s="13" t="str">
-        <x:v>As a Student, I want to view the mentorship slots I created or joined, so that I can track my mentoring activities and commitments.</x:v>
+        <x:v>As a mentorship participant, I want authorized current and historical views so that I can track my activities and commitments.</x:v>
       </x:c>
       <x:c r="J58" s="13" t="str">
-        <x:v>- Student and Alumni mentors see slot series they created.
-- Student mentees see slot series they joined.
-- The next eligible occurrence date/time is shown.
-- Location or meeting link is shown according to mode.
-- Stored slot status and derived FULL/past labels are shown.
-- Historical left, cancelled, and past records remain available where authorized.</x:v>
+        <x:v>- Student and Alumni mentors see series they host; each participant sees their own participation periods and private join message/goals.
+- Ongoing occurrence and the next meeting that has not started are distinct fields.
+- Completed, left, and cancelled periods remain in authorized history; closure does not imply completion.
+- Only the host may retrieve the roster.
+- Meeting links appear only to the host and currently enrolled participants with a remaining ongoing or future meeting.
+- Leaving or historical participation alone cannot reveal the link on detail, list, history, or occurrence-related responses.</x:v>
       </x:c>
       <x:c r="K58" s="15" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="L58" s="15" t="str">
-        <x:v>To Do</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="M58" s="16"/>
       <x:c r="N58" s="16"/>
@@ -63511,9 +63512,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e8b062e2ad248ba"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9989f435867f4f3c"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65850f5ab45c47c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48ae02b4428c43dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66267,7 +66268,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82e35970afbc40de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reafa9bc430ab4583"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66608,7 +66609,7 @@
         <x:v>Mentorship</x:v>
       </x:c>
       <x:c r="C30" s="31" t="str">
-        <x:v>MentorshipSlot supports ONE_TIME, WEEKLY, and BIWEEKLY series with dated MentorshipOccurrences.</x:v>
+        <x:v>ACTIVE, non-anonymized Year-2-or-above Students and ACTIVE, non-anonymized Alumni may register as mentors; mentor availability controls new enrollment, not existing series.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -66619,7 +66620,7 @@
         <x:v>Mentorship</x:v>
       </x:c>
       <x:c r="C31" s="31" t="str">
-        <x:v>One MentorshipEnrollment enrolls an ACTIVE STUDENT in the complete series.</x:v>
+        <x:v>MentorshipSlot supports finite ONE_TIME, WEEKLY, and BIWEEKLY schedules. Asia/Dhaka schedule values generate authoritative dated MentorshipOccurrences; past and ongoing occurrences survive future-only edits and cancellation.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -66630,7 +66631,7 @@
         <x:v>Mentorship</x:v>
       </x:c>
       <x:c r="C32" s="31" t="str">
-        <x:v>Enrollment count, available places, FULL, and past state are derived; historical records are retained.</x:v>
+        <x:v>One active enrollment covers a series' remaining unstarted meetings for an ACTIVE Student or Alumni. Other mentors may enroll, self-enrollment is forbidden, hosted-meeting conflicts block join, and leave/rejoin creates separate retained participation periods.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -66641,7 +66642,7 @@
         <x:v>Career</x:v>
       </x:c>
       <x:c r="C33" s="31" t="str">
-        <x:v>Only ACTIVE ALUMNI users publish JobPosts; no separate alumni-verification state exists.</x:v>
+        <x:v>Enrollment closure, mentor availability, derived FULL, completion, and cancellation are distinct. Counts and vacancies derive from active enrollment; only hosts see rosters, and meeting links are limited to hosts and current participants with a remaining meeting.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -66922,7 +66923,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R182a87bcee8e477d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d62dea8aa394740"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -67413,16 +67414,16 @@
         <x:v>Peer Mentorship</x:v>
       </x:c>
       <x:c r="B15" s="30" t="str">
-        <x:v>DEFERRED</x:v>
+        <x:v>SHOULD</x:v>
       </x:c>
       <x:c r="C15" s="30" t="str">
         <x:v>FR_40–FR_50</x:v>
       </x:c>
       <x:c r="D15" s="30" t="str">
-        <x:v>No one-month commitment</x:v>
+        <x:v>Backend lifecycle corrections in progress: finite occurrences, enrollment periods, conflict/capacity serialization, privacy-safe responses, and retained history</x:v>
       </x:c>
       <x:c r="E15" s="30" t="str">
-        <x:v>Retained in the product baseline for later implementation.</x:v>
+        <x:v>Flutter remains on existing endpoint shapes where practical. Reopen and history fields/endpoints are additive; cross-module search, complete anonymization, and the dedicated notification-target resolver remain deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="36" hidden="0" customHeight="1">
@@ -67476,7 +67477,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R228a155841304b98"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffb473c9d31a458a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>